<commit_message>
Prepped for lin fit
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=3.xlsx
+++ b/Fit Results/AllFitsF1=3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wolfw\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95537571-7E03-4A8C-BE2E-D6F4B610A6AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="10992" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Together" sheetId="1" r:id="rId1"/>
@@ -30,9 +30,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -3263,6 +3260,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3270,7 +3268,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5901,6 +5898,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5908,7 +5906,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9084,6 +9081,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9091,7 +9089,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9585,6 +9582,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9592,7 +9590,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12153,6 +12150,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12160,7 +12158,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12654,6 +12651,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12661,7 +12659,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16527,12 +16524,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R297"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -16550,7 +16547,7 @@
       </c>
       <c r="R1" s="1"/>
     </row>
-    <row r="2" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -16572,7 +16569,7 @@
         <v>4.2703475132141157E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -16594,7 +16591,7 @@
         <v>0.18809412531311234</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -16606,7 +16603,7 @@
       </c>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -16628,7 +16625,7 @@
         <v>0.22378459935658199</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -16650,7 +16647,7 @@
         <v>0.228434718604688</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -16672,7 +16669,7 @@
         <v>0.221372998488612</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -16694,7 +16691,7 @@
         <v>0.225975457594905</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
@@ -16716,7 +16713,7 @@
         <v>0.225216837741747</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="1" t="s">
         <v>309</v>
       </c>
@@ -16738,7 +16735,7 @@
         <v>0.229746279532067</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
         <v>310</v>
       </c>
@@ -16760,7 +16757,7 @@
         <v>0.22722518963626401</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -16782,7 +16779,7 @@
         <v>0.222965184868961</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1" t="s">
         <v>311</v>
       </c>
@@ -16804,7 +16801,7 @@
         <v>0.22898718060617901</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -16815,7 +16812,7 @@
         <v>0.13498234565869699</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -16826,7 +16823,7 @@
         <v>0.13854180631109</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -16837,7 +16834,7 @@
         <v>0.13743837454275501</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -16848,7 +16845,7 @@
         <v>0.13738267695902801</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
@@ -16859,7 +16856,7 @@
         <v>0.14159428045373601</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
@@ -16870,7 +16867,7 @@
         <v>0.14232784705226301</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1" t="s">
         <v>13</v>
       </c>
@@ -16881,7 +16878,7 @@
         <v>0.14391242117178599</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
@@ -16892,7 +16889,7 @@
         <v>0.13920272125085101</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="1" t="s">
         <v>15</v>
       </c>
@@ -16903,7 +16900,7 @@
         <v>0.14459533841685501</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="1" t="s">
         <v>312</v>
       </c>
@@ -16914,7 +16911,7 @@
         <v>0.13915991329959099</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="1" t="s">
         <v>16</v>
       </c>
@@ -16925,7 +16922,7 @@
         <v>0.144975058104169</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
@@ -16936,7 +16933,7 @@
         <v>0.14496624110967199</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1" t="s">
         <v>18</v>
       </c>
@@ -16947,7 +16944,7 @@
         <v>0.14341121488491801</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
         <v>19</v>
       </c>
@@ -16958,7 +16955,7 @@
         <v>0.14388771373763901</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1" t="s">
         <v>20</v>
       </c>
@@ -16969,7 +16966,7 @@
         <v>0.14091026017191899</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1" t="s">
         <v>313</v>
       </c>
@@ -16980,7 +16977,7 @@
         <v>0.13928443937518301</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="1" t="s">
         <v>21</v>
       </c>
@@ -16991,7 +16988,7 @@
         <v>0.14449758570660601</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
         <v>314</v>
       </c>
@@ -17002,7 +16999,7 @@
         <v>0.14272080636913501</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="1" t="s">
         <v>315</v>
       </c>
@@ -17013,7 +17010,7 @@
         <v>0.14380448214622399</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1" t="s">
         <v>22</v>
       </c>
@@ -17024,7 +17021,7 @@
         <v>0.13910873933717599</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
         <v>28</v>
       </c>
@@ -17035,7 +17032,7 @@
         <v>0.117218052017694</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="1" t="s">
         <v>29</v>
       </c>
@@ -17046,7 +17043,7 @@
         <v>0.116738218899043</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="1" t="s">
         <v>30</v>
       </c>
@@ -17057,7 +17054,7 @@
         <v>0.116641895814922</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="1" t="s">
         <v>31</v>
       </c>
@@ -17068,7 +17065,7 @@
         <v>0.117986722306339</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="1" t="s">
         <v>32</v>
       </c>
@@ -17079,7 +17076,7 @@
         <v>0.116363944216263</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="1" t="s">
         <v>33</v>
       </c>
@@ -17090,7 +17087,7 @@
         <v>0.117960737624138</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="1" t="s">
         <v>34</v>
       </c>
@@ -17101,7 +17098,7 @@
         <v>0.11777189549636199</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="1" t="s">
         <v>35</v>
       </c>
@@ -17112,7 +17109,7 @@
         <v>0.118362346500101</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="1" t="s">
         <v>36</v>
       </c>
@@ -17123,7 +17120,7 @@
         <v>0.11875028071223</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="1" t="s">
         <v>37</v>
       </c>
@@ -17134,7 +17131,7 @@
         <v>0.118209453954305</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="1" t="s">
         <v>38</v>
       </c>
@@ -17145,7 +17142,7 @@
         <v>0.116577694816434</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="1" t="s">
         <v>39</v>
       </c>
@@ -17156,7 +17153,7 @@
         <v>0.117670638852321</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="1" t="s">
         <v>40</v>
       </c>
@@ -17167,7 +17164,7 @@
         <v>0.118098845799444</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="1" t="s">
         <v>41</v>
       </c>
@@ -17178,7 +17175,7 @@
         <v>0.11655919684067299</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="1" t="s">
         <v>42</v>
       </c>
@@ -17189,7 +17186,7 @@
         <v>0.118487075826876</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="1" t="s">
         <v>43</v>
       </c>
@@ -17200,7 +17197,7 @@
         <v>0.117049111989703</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="1" t="s">
         <v>44</v>
       </c>
@@ -17211,7 +17208,7 @@
         <v>0.116964493443121</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="1" t="s">
         <v>45</v>
       </c>
@@ -17222,7 +17219,7 @@
         <v>0.1174932059815</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="1" t="s">
         <v>46</v>
       </c>
@@ -17233,7 +17230,7 @@
         <v>0.118724780988732</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="1" t="s">
         <v>47</v>
       </c>
@@ -17244,7 +17241,7 @@
         <v>0.11857414162119</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="1" t="s">
         <v>48</v>
       </c>
@@ -17255,7 +17252,7 @@
         <v>0.116857985488521</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="1" t="s">
         <v>49</v>
       </c>
@@ -17266,7 +17263,7 @@
         <v>0.117839930521939</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="1" t="s">
         <v>50</v>
       </c>
@@ -17277,7 +17274,7 @@
         <v>0.116123290748398</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="1" t="s">
         <v>51</v>
       </c>
@@ -17288,7 +17285,7 @@
         <v>0.116339626646247</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="1" t="s">
         <v>52</v>
       </c>
@@ -17299,7 +17296,7 @@
         <v>0.118521454357363</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="1" t="s">
         <v>53</v>
       </c>
@@ -17310,7 +17307,7 @@
         <v>0.117743388207075</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="1" t="s">
         <v>54</v>
       </c>
@@ -17321,7 +17318,7 @@
         <v>0.116823099810358</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="1" t="s">
         <v>55</v>
       </c>
@@ -17332,7 +17329,7 @@
         <v>0.118509294607666</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="1" t="s">
         <v>56</v>
       </c>
@@ -17343,7 +17340,7 @@
         <v>0.118631007440724</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="1" t="s">
         <v>57</v>
       </c>
@@ -17354,7 +17351,7 @@
         <v>0.117484320873481</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="1" t="s">
         <v>58</v>
       </c>
@@ -17365,7 +17362,7 @@
         <v>0.118251546607688</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="1" t="s">
         <v>59</v>
       </c>
@@ -17376,7 +17373,7 @@
         <v>0.118181098472526</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="1" t="s">
         <v>60</v>
       </c>
@@ -17387,7 +17384,7 @@
         <v>8.9287039240001795E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="1" t="s">
         <v>61</v>
       </c>
@@ -17398,7 +17395,7 @@
         <v>8.9953273584561996E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="1" t="s">
         <v>62</v>
       </c>
@@ -17409,7 +17406,7 @@
         <v>9.1230909809772498E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="1" t="s">
         <v>63</v>
       </c>
@@ -17420,7 +17417,7 @@
         <v>9.0037965159722497E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="1" t="s">
         <v>64</v>
       </c>
@@ -17431,7 +17428,7 @@
         <v>9.2063662732121604E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="1" t="s">
         <v>65</v>
       </c>
@@ -17442,7 +17439,7 @@
         <v>9.0566169869859395E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="1" t="s">
         <v>66</v>
       </c>
@@ -17453,7 +17450,7 @@
         <v>9.1281359996997199E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="1" t="s">
         <v>67</v>
       </c>
@@ -17464,7 +17461,7 @@
         <v>9.0246189977935598E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="1" t="s">
         <v>68</v>
       </c>
@@ -17475,7 +17472,7 @@
         <v>8.7987770056780296E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="1" t="s">
         <v>69</v>
       </c>
@@ -17486,7 +17483,7 @@
         <v>9.1038024594974204E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="1" t="s">
         <v>70</v>
       </c>
@@ -17497,7 +17494,7 @@
         <v>9.0356969610468907E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="1" t="s">
         <v>71</v>
       </c>
@@ -17508,7 +17505,7 @@
         <v>8.9055177802521202E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" s="1" t="s">
         <v>72</v>
       </c>
@@ -17519,7 +17516,7 @@
         <v>9.0556231765949805E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" s="1" t="s">
         <v>73</v>
       </c>
@@ -17530,7 +17527,7 @@
         <v>9.1259865204828206E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" s="1" t="s">
         <v>74</v>
       </c>
@@ -17541,7 +17538,7 @@
         <v>8.8371089308141498E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" s="1" t="s">
         <v>75</v>
       </c>
@@ -17552,7 +17549,7 @@
         <v>8.9886315679026302E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" s="1" t="s">
         <v>76</v>
       </c>
@@ -17563,7 +17560,7 @@
         <v>0.22378459935658199</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" s="1" t="s">
         <v>77</v>
       </c>
@@ -17574,7 +17571,7 @@
         <v>0.228434718604688</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" s="1" t="s">
         <v>78</v>
       </c>
@@ -17585,7 +17582,7 @@
         <v>0.221372998488612</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" s="1" t="s">
         <v>79</v>
       </c>
@@ -17596,7 +17593,7 @@
         <v>0.225975457594905</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" s="1" t="s">
         <v>80</v>
       </c>
@@ -17607,7 +17604,7 @@
         <v>0.225216837741747</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" s="1" t="s">
         <v>81</v>
       </c>
@@ -17618,7 +17615,7 @@
         <v>0.229746279532067</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" s="1" t="s">
         <v>82</v>
       </c>
@@ -17629,7 +17626,7 @@
         <v>0.22722518963626401</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" s="1" t="s">
         <v>83</v>
       </c>
@@ -17640,7 +17637,7 @@
         <v>0.222965184868961</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" s="1" t="s">
         <v>84</v>
       </c>
@@ -17651,7 +17648,7 @@
         <v>0.22898718060617901</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" s="1" t="s">
         <v>85</v>
       </c>
@@ -17662,7 +17659,7 @@
         <v>0.22580668748875701</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" s="1" t="s">
         <v>86</v>
       </c>
@@ -17673,7 +17670,7 @@
         <v>0.231594890582631</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A93" s="1" t="s">
         <v>87</v>
       </c>
@@ -17684,7 +17681,7 @@
         <v>0.224583618990919</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" s="1" t="s">
         <v>88</v>
       </c>
@@ -17695,7 +17692,7 @@
         <v>0.23249128317182099</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" s="1" t="s">
         <v>89</v>
       </c>
@@ -17706,7 +17703,7 @@
         <v>0.23073510515949899</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" s="1" t="s">
         <v>90</v>
       </c>
@@ -17717,7 +17714,7 @@
         <v>0.229179326874075</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" s="1" t="s">
         <v>91</v>
       </c>
@@ -17728,7 +17725,7 @@
         <v>0.226024665246639</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A98" s="1" t="s">
         <v>92</v>
       </c>
@@ -17739,7 +17736,7 @@
         <v>0.22988414195496401</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A99" s="1" t="s">
         <v>93</v>
       </c>
@@ -17750,7 +17747,7 @@
         <v>0.22795719930278499</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A100" s="1" t="s">
         <v>94</v>
       </c>
@@ -17761,7 +17758,7 @@
         <v>0.227267035209756</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A101" s="1" t="s">
         <v>95</v>
       </c>
@@ -17772,7 +17769,7 @@
         <v>0.22728875634974799</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A102" s="1" t="s">
         <v>96</v>
       </c>
@@ -17783,7 +17780,7 @@
         <v>0.22819660608103401</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A103" s="1" t="s">
         <v>97</v>
       </c>
@@ -17794,7 +17791,7 @@
         <v>0.22449918198189101</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A104" s="1" t="s">
         <v>98</v>
       </c>
@@ -17805,7 +17802,7 @@
         <v>0.22352994908158599</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" s="1" t="s">
         <v>99</v>
       </c>
@@ -17816,7 +17813,7 @@
         <v>0.22753327784977401</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A106" s="1" t="s">
         <v>100</v>
       </c>
@@ -17827,7 +17824,7 @@
         <v>0.22784419865740199</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A107" s="1" t="s">
         <v>101</v>
       </c>
@@ -17838,7 +17835,7 @@
         <v>0.225433003733543</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A108" s="1" t="s">
         <v>102</v>
       </c>
@@ -17849,7 +17846,7 @@
         <v>0.22712348211729699</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A109" s="1" t="s">
         <v>103</v>
       </c>
@@ -17860,7 +17857,7 @@
         <v>0.22894109101944199</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A110" s="1" t="s">
         <v>104</v>
       </c>
@@ -17871,7 +17868,7 @@
         <v>0.23027592968354901</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A111" s="1" t="s">
         <v>105</v>
       </c>
@@ -17882,7 +17879,7 @@
         <v>0.22733899516780401</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A112" s="1" t="s">
         <v>106</v>
       </c>
@@ -17893,7 +17890,7 @@
         <v>0.22718964047891599</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" s="1" t="s">
         <v>107</v>
       </c>
@@ -17904,7 +17901,7 @@
         <v>0.22249606599096799</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A114" s="1" t="s">
         <v>108</v>
       </c>
@@ -17915,7 +17912,7 @@
         <v>0.22770140189949001</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A115" s="1" t="s">
         <v>109</v>
       </c>
@@ -17926,7 +17923,7 @@
         <v>0.22467693879523801</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A116" s="1" t="s">
         <v>110</v>
       </c>
@@ -17937,7 +17934,7 @@
         <v>0.22590951148508701</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A117" s="1" t="s">
         <v>111</v>
       </c>
@@ -17948,7 +17945,7 @@
         <v>0.22795873224990801</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A118" s="1" t="s">
         <v>112</v>
       </c>
@@ -17959,7 +17956,7 @@
         <v>0.26064960163891099</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A119" s="1" t="s">
         <v>113</v>
       </c>
@@ -17970,7 +17967,7 @@
         <v>0.25338188968269398</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A120" s="1" t="s">
         <v>114</v>
       </c>
@@ -17981,7 +17978,7 @@
         <v>0.25038094455952498</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A121" s="1" t="s">
         <v>115</v>
       </c>
@@ -17992,7 +17989,7 @@
         <v>0.256215228918099</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" s="1" t="s">
         <v>116</v>
       </c>
@@ -18003,7 +18000,7 @@
         <v>0.25483329669185101</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A123" s="1" t="s">
         <v>117</v>
       </c>
@@ -18014,7 +18011,7 @@
         <v>0.25854387484878599</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A124" s="1" t="s">
         <v>118</v>
       </c>
@@ -18025,7 +18022,7 @@
         <v>0.25519336396030601</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A125" s="1" t="s">
         <v>119</v>
       </c>
@@ -18036,7 +18033,7 @@
         <v>0.25663303680948102</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A126" s="1" t="s">
         <v>120</v>
       </c>
@@ -18047,7 +18044,7 @@
         <v>0.25601459599486398</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A127" s="1" t="s">
         <v>121</v>
       </c>
@@ -18058,7 +18055,7 @@
         <v>0.25648553124648299</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A128" s="1" t="s">
         <v>122</v>
       </c>
@@ -18069,7 +18066,7 @@
         <v>0.25339182435774998</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A129" s="1" t="s">
         <v>123</v>
       </c>
@@ -18080,7 +18077,7 @@
         <v>0.26261256236820102</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A130" s="1" t="s">
         <v>124</v>
       </c>
@@ -18091,7 +18088,7 @@
         <v>0.25914013258546797</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A131" s="1" t="s">
         <v>125</v>
       </c>
@@ -18102,7 +18099,7 @@
         <v>0.25187380012057398</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A132" s="1" t="s">
         <v>126</v>
       </c>
@@ -18113,7 +18110,7 @@
         <v>0.25861462842520899</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A133" s="1" t="s">
         <v>127</v>
       </c>
@@ -18124,7 +18121,7 @@
         <v>0.26412000142144099</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A134" s="1" t="s">
         <v>128</v>
       </c>
@@ -18135,7 +18132,7 @@
         <v>0.25505739125523702</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A135" s="1" t="s">
         <v>129</v>
       </c>
@@ -18146,7 +18143,7 @@
         <v>0.25268334549192301</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A136" s="1" t="s">
         <v>130</v>
       </c>
@@ -18157,7 +18154,7 @@
         <v>0.254203134019032</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A137" s="1" t="s">
         <v>131</v>
       </c>
@@ -18168,7 +18165,7 @@
         <v>0.25355249186689299</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A138" s="1" t="s">
         <v>132</v>
       </c>
@@ -18179,7 +18176,7 @@
         <v>0.258640908855092</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A139" s="1" t="s">
         <v>133</v>
       </c>
@@ -18190,7 +18187,7 @@
         <v>0.25176887581155899</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A140" s="1" t="s">
         <v>134</v>
       </c>
@@ -18201,7 +18198,7 @@
         <v>0.25436276153236997</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A141" s="1" t="s">
         <v>135</v>
       </c>
@@ -18212,7 +18209,7 @@
         <v>0.25848980394328103</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A142" s="1" t="s">
         <v>136</v>
       </c>
@@ -18223,7 +18220,7 @@
         <v>0.25493042534243598</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A143" s="1" t="s">
         <v>137</v>
       </c>
@@ -18234,7 +18231,7 @@
         <v>0.25702073078272197</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A144" s="1" t="s">
         <v>138</v>
       </c>
@@ -18245,7 +18242,7 @@
         <v>0.25281370286486299</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A145" s="1" t="s">
         <v>139</v>
       </c>
@@ -18256,7 +18253,7 @@
         <v>0.25787828139437702</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A146" s="1" t="s">
         <v>140</v>
       </c>
@@ -18267,7 +18264,7 @@
         <v>0.255030114263046</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A147" s="1" t="s">
         <v>141</v>
       </c>
@@ -18278,7 +18275,7 @@
         <v>0.25326708245889501</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A148" s="1" t="s">
         <v>142</v>
       </c>
@@ -18289,7 +18286,7 @@
         <v>0.25901851572451601</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A149" s="1" t="s">
         <v>143</v>
       </c>
@@ -18300,7 +18297,7 @@
         <v>0.25402214979933802</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A150" s="1" t="s">
         <v>144</v>
       </c>
@@ -18311,7 +18308,7 @@
         <v>0.25207440807669201</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A151" s="1" t="s">
         <v>145</v>
       </c>
@@ -18322,7 +18319,7 @@
         <v>0.25648835225167999</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A152" s="1" t="s">
         <v>146</v>
       </c>
@@ -18333,7 +18330,7 @@
         <v>0.25619702232418301</v>
       </c>
     </row>
-    <row r="153" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A153" s="1" t="s">
         <v>147</v>
       </c>
@@ -18344,7 +18341,7 @@
         <v>0.256904989972564</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A154" s="1" t="s">
         <v>148</v>
       </c>
@@ -18355,7 +18352,7 @@
         <v>0.25656545981822299</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A155" s="1" t="s">
         <v>149</v>
       </c>
@@ -18366,7 +18363,7 @@
         <v>0.25471437628790899</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A156" s="1" t="s">
         <v>150</v>
       </c>
@@ -18377,7 +18374,7 @@
         <v>0.25564492601438199</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A157" s="1" t="s">
         <v>151</v>
       </c>
@@ -18388,7 +18385,7 @@
         <v>0.26266359379455601</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A158" s="1" t="s">
         <v>152</v>
       </c>
@@ -18399,7 +18396,7 @@
         <v>0.25914186884267898</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A159" s="1" t="s">
         <v>153</v>
       </c>
@@ -18410,7 +18407,7 @@
         <v>0.25621155685651098</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A160" s="1" t="s">
         <v>154</v>
       </c>
@@ -18421,7 +18418,7 @@
         <v>0.25866494788723898</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A161" s="1" t="s">
         <v>155</v>
       </c>
@@ -18432,7 +18429,7 @@
         <v>0.25801756322347102</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A162" s="1" t="s">
         <v>156</v>
       </c>
@@ -18443,7 +18440,7 @@
         <v>0.25944545650678502</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A163" s="1" t="s">
         <v>157</v>
       </c>
@@ -18454,7 +18451,7 @@
         <v>0.25336488450504602</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A164" s="1" t="s">
         <v>158</v>
       </c>
@@ -18465,7 +18462,7 @@
         <v>0.261553420142073</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A165" s="1" t="s">
         <v>159</v>
       </c>
@@ -18476,7 +18473,7 @@
         <v>0.26019522603942802</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A166" s="1" t="s">
         <v>160</v>
       </c>
@@ -18487,7 +18484,7 @@
         <v>0.25868729407005198</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A167" s="1" t="s">
         <v>161</v>
       </c>
@@ -18498,7 +18495,7 @@
         <v>0.25516460879894798</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A168" s="1" t="s">
         <v>162</v>
       </c>
@@ -18509,7 +18506,7 @@
         <v>0.25295075090609098</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A169" s="1" t="s">
         <v>163</v>
       </c>
@@ -18520,7 +18517,7 @@
         <v>0.256452611497334</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A170" s="1" t="s">
         <v>164</v>
       </c>
@@ -18531,7 +18528,7 @@
         <v>0.25868777299010298</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A171" s="1" t="s">
         <v>165</v>
       </c>
@@ -18542,7 +18539,7 @@
         <v>0.2539674766801</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A172" s="1" t="s">
         <v>166</v>
       </c>
@@ -18553,7 +18550,7 @@
         <v>0.17294771128421699</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A173" s="1" t="s">
         <v>167</v>
       </c>
@@ -18564,7 +18561,7 @@
         <v>0.175665485735155</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A174" s="1" t="s">
         <v>168</v>
       </c>
@@ -18575,7 +18572,7 @@
         <v>0.17382778027635701</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A175" s="1" t="s">
         <v>169</v>
       </c>
@@ -18586,7 +18583,7 @@
         <v>0.17455983570099701</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A176" s="1" t="s">
         <v>170</v>
       </c>
@@ -18597,7 +18594,7 @@
         <v>0.17664296551393399</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A177" s="1" t="s">
         <v>171</v>
       </c>
@@ -18608,7 +18605,7 @@
         <v>0.17708531560420199</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A178" s="1" t="s">
         <v>172</v>
       </c>
@@ -18619,7 +18616,7 @@
         <v>0.17557573140333699</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A179" s="1" t="s">
         <v>173</v>
       </c>
@@ -18630,7 +18627,7 @@
         <v>0.173457649972002</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A180" s="1" t="s">
         <v>174</v>
       </c>
@@ -18641,7 +18638,7 @@
         <v>0.17535865105134299</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A181" s="1" t="s">
         <v>175</v>
       </c>
@@ -18652,7 +18649,7 @@
         <v>0.175039518424147</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A182" s="1" t="s">
         <v>176</v>
       </c>
@@ -18663,7 +18660,7 @@
         <v>0.17459939950666101</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A183" s="1" t="s">
         <v>177</v>
       </c>
@@ -18674,7 +18671,7 @@
         <v>0.17177387798819599</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A184" s="1" t="s">
         <v>178</v>
       </c>
@@ -18685,7 +18682,7 @@
         <v>0.172049396498035</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A185" s="1" t="s">
         <v>179</v>
       </c>
@@ -18696,7 +18693,7 @@
         <v>0.17416028353340501</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A186" s="1" t="s">
         <v>180</v>
       </c>
@@ -18707,7 +18704,7 @@
         <v>0.17432866559164001</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A187" s="1" t="s">
         <v>181</v>
       </c>
@@ -18718,7 +18715,7 @@
         <v>0.17371638201273101</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A188" s="1" t="s">
         <v>182</v>
       </c>
@@ -18729,7 +18726,7 @@
         <v>0.17123203171632401</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A189" s="1" t="s">
         <v>183</v>
       </c>
@@ -18740,7 +18737,7 @@
         <v>0.17318569822136001</v>
       </c>
     </row>
-    <row r="190" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A190" s="1" t="s">
         <v>184</v>
       </c>
@@ -18751,7 +18748,7 @@
         <v>0.17669669700448201</v>
       </c>
     </row>
-    <row r="191" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A191" s="1" t="s">
         <v>185</v>
       </c>
@@ -18762,7 +18759,7 @@
         <v>0.17723933870696301</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A192" s="1" t="s">
         <v>186</v>
       </c>
@@ -18773,7 +18770,7 @@
         <v>0.17063092731327101</v>
       </c>
     </row>
-    <row r="193" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A193" s="1" t="s">
         <v>187</v>
       </c>
@@ -18784,7 +18781,7 @@
         <v>0.17490193092626999</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A194" s="1" t="s">
         <v>188</v>
       </c>
@@ -18795,7 +18792,7 @@
         <v>0.17702310390171999</v>
       </c>
     </row>
-    <row r="195" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A195" s="1" t="s">
         <v>189</v>
       </c>
@@ -18806,7 +18803,7 @@
         <v>0.171948853936535</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A196" s="1" t="s">
         <v>190</v>
       </c>
@@ -18817,7 +18814,7 @@
         <v>0.17411860264206899</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A197" s="1" t="s">
         <v>191</v>
       </c>
@@ -18828,7 +18825,7 @@
         <v>0.175935205113702</v>
       </c>
     </row>
-    <row r="198" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A198" s="1" t="s">
         <v>192</v>
       </c>
@@ -18839,7 +18836,7 @@
         <v>0.17427622300988699</v>
       </c>
     </row>
-    <row r="199" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A199" s="1" t="s">
         <v>193</v>
       </c>
@@ -18850,7 +18847,7 @@
         <v>0.17224969239811899</v>
       </c>
     </row>
-    <row r="200" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A200" s="1" t="s">
         <v>194</v>
       </c>
@@ -18861,7 +18858,7 @@
         <v>0.17435257559575301</v>
       </c>
     </row>
-    <row r="201" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A201" s="1" t="s">
         <v>195</v>
       </c>
@@ -18872,7 +18869,7 @@
         <v>0.171222354567128</v>
       </c>
     </row>
-    <row r="202" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A202" s="1" t="s">
         <v>196</v>
       </c>
@@ -18883,7 +18880,7 @@
         <v>0.17230494746765301</v>
       </c>
     </row>
-    <row r="203" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A203" s="1" t="s">
         <v>197</v>
       </c>
@@ -18894,7 +18891,7 @@
         <v>0.17976030708667101</v>
       </c>
     </row>
-    <row r="204" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A204" s="1" t="s">
         <v>198</v>
       </c>
@@ -18905,7 +18902,7 @@
         <v>0.174433801903358</v>
       </c>
     </row>
-    <row r="205" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A205" s="1" t="s">
         <v>199</v>
       </c>
@@ -18916,7 +18913,7 @@
         <v>0.17714435708530099</v>
       </c>
     </row>
-    <row r="206" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A206" s="1" t="s">
         <v>200</v>
       </c>
@@ -18927,7 +18924,7 @@
         <v>0.17086804073973499</v>
       </c>
     </row>
-    <row r="207" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A207" s="1" t="s">
         <v>201</v>
       </c>
@@ -18938,7 +18935,7 @@
         <v>0.171697248433512</v>
       </c>
     </row>
-    <row r="208" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A208" s="1" t="s">
         <v>202</v>
       </c>
@@ -18949,7 +18946,7 @@
         <v>0.17443666559002999</v>
       </c>
     </row>
-    <row r="209" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A209" s="1" t="s">
         <v>203</v>
       </c>
@@ -18960,7 +18957,7 @@
         <v>0.17690051952166999</v>
       </c>
     </row>
-    <row r="210" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A210" s="1" t="s">
         <v>204</v>
       </c>
@@ -18971,19 +18968,19 @@
         <v>0.17654554655181801</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
     </row>
-    <row r="214" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A214" s="1" t="s">
         <v>245</v>
       </c>
@@ -18994,7 +18991,7 @@
         <v>0.21689563024651701</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A215" s="1" t="s">
         <v>246</v>
       </c>
@@ -19005,7 +19002,7 @@
         <v>0.21250705902688999</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A216" s="1" t="s">
         <v>247</v>
       </c>
@@ -19016,7 +19013,7 @@
         <v>0.21268324019514501</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A217" s="1" t="s">
         <v>248</v>
       </c>
@@ -19027,7 +19024,7 @@
         <v>0.21049345542616399</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A218" s="1" t="s">
         <v>249</v>
       </c>
@@ -19038,7 +19035,7 @@
         <v>0.214431740824571</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A219" s="1" t="s">
         <v>250</v>
       </c>
@@ -19049,7 +19046,7 @@
         <v>0.21026943516751501</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A220" s="1" t="s">
         <v>251</v>
       </c>
@@ -19060,7 +19057,7 @@
         <v>0.211983108185162</v>
       </c>
     </row>
-    <row r="221" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A221" s="1" t="s">
         <v>252</v>
       </c>
@@ -19071,7 +19068,7 @@
         <v>0.212540414406241</v>
       </c>
     </row>
-    <row r="222" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A222" s="1" t="s">
         <v>253</v>
       </c>
@@ -19082,7 +19079,7 @@
         <v>0.21316933311979799</v>
       </c>
     </row>
-    <row r="223" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A223" s="1" t="s">
         <v>254</v>
       </c>
@@ -19093,7 +19090,7 @@
         <v>0.212515123863107</v>
       </c>
     </row>
-    <row r="224" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A224" s="1" t="s">
         <v>255</v>
       </c>
@@ -19104,7 +19101,7 @@
         <v>0.21030240285409901</v>
       </c>
     </row>
-    <row r="225" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A225" s="1" t="s">
         <v>256</v>
       </c>
@@ -19115,7 +19112,7 @@
         <v>0.213000429148374</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A226" s="1" t="s">
         <v>257</v>
       </c>
@@ -19126,7 +19123,7 @@
         <v>0.21204120218539499</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A227" s="1" t="s">
         <v>258</v>
       </c>
@@ -19137,7 +19134,7 @@
         <v>0.211005527878392</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A228" s="1" t="s">
         <v>259</v>
       </c>
@@ -19148,7 +19145,7 @@
         <v>0.21490935202097999</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A229" s="1" t="s">
         <v>260</v>
       </c>
@@ -19159,7 +19156,7 @@
         <v>0.214705500945685</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A230" s="1" t="s">
         <v>261</v>
       </c>
@@ -19170,7 +19167,7 @@
         <v>0.21046954774395399</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A231" s="1" t="s">
         <v>262</v>
       </c>
@@ -19181,7 +19178,7 @@
         <v>0.212979730482002</v>
       </c>
     </row>
-    <row r="232" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A232" s="1" t="s">
         <v>263</v>
       </c>
@@ -19192,7 +19189,7 @@
         <v>0.21145441547031901</v>
       </c>
     </row>
-    <row r="233" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A233" s="1" t="s">
         <v>264</v>
       </c>
@@ -19203,7 +19200,7 @@
         <v>0.21334229216903</v>
       </c>
     </row>
-    <row r="234" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A234" s="1" t="s">
         <v>265</v>
       </c>
@@ -19214,7 +19211,7 @@
         <v>0.21313225436689001</v>
       </c>
     </row>
-    <row r="235" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A235" s="1" t="s">
         <v>266</v>
       </c>
@@ -19225,7 +19222,7 @@
         <v>0.21364986681269199</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A236" s="1" t="s">
         <v>267</v>
       </c>
@@ -19236,7 +19233,7 @@
         <v>0.21046298569896901</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A237" s="1" t="s">
         <v>268</v>
       </c>
@@ -19247,7 +19244,7 @@
         <v>0.21370475343700501</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A238" s="1" t="s">
         <v>269</v>
       </c>
@@ -19258,7 +19255,7 @@
         <v>0.213427613164866</v>
       </c>
     </row>
-    <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A239" s="1" t="s">
         <v>270</v>
       </c>
@@ -19269,7 +19266,7 @@
         <v>0.21285885222227299</v>
       </c>
     </row>
-    <row r="240" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A240" s="1" t="s">
         <v>271</v>
       </c>
@@ -19280,7 +19277,7 @@
         <v>0.21229610722325801</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A241" s="1" t="s">
         <v>272</v>
       </c>
@@ -19291,7 +19288,7 @@
         <v>0.213479995323273</v>
       </c>
     </row>
-    <row r="242" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A242" s="1" t="s">
         <v>244</v>
       </c>
@@ -19302,7 +19299,7 @@
         <v>0.23747635372092801</v>
       </c>
     </row>
-    <row r="243" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A243" s="1" t="s">
         <v>220</v>
       </c>
@@ -19313,7 +19310,7 @@
         <v>0.24180291421483799</v>
       </c>
     </row>
-    <row r="244" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A244" s="1" t="s">
         <v>221</v>
       </c>
@@ -19324,7 +19321,7 @@
         <v>0.23775144209915899</v>
       </c>
     </row>
-    <row r="245" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A245" s="1" t="s">
         <v>222</v>
       </c>
@@ -19335,7 +19332,7 @@
         <v>0.24065215342237201</v>
       </c>
     </row>
-    <row r="246" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A246" s="1" t="s">
         <v>223</v>
       </c>
@@ -19346,7 +19343,7 @@
         <v>0.238634580986853</v>
       </c>
     </row>
-    <row r="247" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A247" s="1" t="s">
         <v>224</v>
       </c>
@@ -19357,7 +19354,7 @@
         <v>0.24123516367901099</v>
       </c>
     </row>
-    <row r="248" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A248" s="1" t="s">
         <v>225</v>
       </c>
@@ -19368,7 +19365,7 @@
         <v>0.23838761262462899</v>
       </c>
     </row>
-    <row r="249" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A249" s="1" t="s">
         <v>226</v>
       </c>
@@ -19379,7 +19376,7 @@
         <v>0.23787175668006799</v>
       </c>
     </row>
-    <row r="250" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A250" s="1" t="s">
         <v>227</v>
       </c>
@@ -19390,7 +19387,7 @@
         <v>0.235957408677299</v>
       </c>
     </row>
-    <row r="251" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A251" s="1" t="s">
         <v>228</v>
       </c>
@@ -19401,7 +19398,7 @@
         <v>0.23761103430247099</v>
       </c>
     </row>
-    <row r="252" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A252" s="1" t="s">
         <v>229</v>
       </c>
@@ -19412,7 +19409,7 @@
         <v>0.24049928819975</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A253" s="1" t="s">
         <v>230</v>
       </c>
@@ -19423,7 +19420,7 @@
         <v>0.23875237313230799</v>
       </c>
     </row>
-    <row r="254" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A254" s="1" t="s">
         <v>231</v>
       </c>
@@ -19434,7 +19431,7 @@
         <v>0.23577509684512599</v>
       </c>
     </row>
-    <row r="255" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A255" s="1" t="s">
         <v>232</v>
       </c>
@@ -19445,7 +19442,7 @@
         <v>0.23798590162913699</v>
       </c>
     </row>
-    <row r="256" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A256" s="1" t="s">
         <v>233</v>
       </c>
@@ -19456,7 +19453,7 @@
         <v>0.23776270729380899</v>
       </c>
     </row>
-    <row r="257" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A257" s="1" t="s">
         <v>234</v>
       </c>
@@ -19467,7 +19464,7 @@
         <v>0.23525871098023601</v>
       </c>
     </row>
-    <row r="258" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A258" s="1" t="s">
         <v>235</v>
       </c>
@@ -19478,7 +19475,7 @@
         <v>0.23822698567085801</v>
       </c>
     </row>
-    <row r="259" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A259" s="1" t="s">
         <v>236</v>
       </c>
@@ -19489,7 +19486,7 @@
         <v>0.236137249858582</v>
       </c>
     </row>
-    <row r="260" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A260" s="1" t="s">
         <v>237</v>
       </c>
@@ -19500,7 +19497,7 @@
         <v>0.236589149526167</v>
       </c>
     </row>
-    <row r="261" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A261" s="1" t="s">
         <v>238</v>
       </c>
@@ -19511,7 +19508,7 @@
         <v>0.234995035195148</v>
       </c>
     </row>
-    <row r="262" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A262" s="1" t="s">
         <v>239</v>
       </c>
@@ -19522,7 +19519,7 @@
         <v>0.238435257488993</v>
       </c>
     </row>
-    <row r="263" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A263" s="1" t="s">
         <v>240</v>
       </c>
@@ -19533,7 +19530,7 @@
         <v>0.23631298859917599</v>
       </c>
     </row>
-    <row r="264" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A264" s="1" t="s">
         <v>241</v>
       </c>
@@ -19544,7 +19541,7 @@
         <v>0.238968925765909</v>
       </c>
     </row>
-    <row r="265" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A265" s="1" t="s">
         <v>242</v>
       </c>
@@ -19555,7 +19552,7 @@
         <v>0.237506075673066</v>
       </c>
     </row>
-    <row r="266" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A266" s="1" t="s">
         <v>243</v>
       </c>
@@ -19566,7 +19563,7 @@
         <v>0.237718713583811</v>
       </c>
     </row>
-    <row r="267" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A267" s="1" t="s">
         <v>276</v>
       </c>
@@ -19577,7 +19574,7 @@
         <v>0.29193451692567801</v>
       </c>
     </row>
-    <row r="268" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A268" s="1" t="s">
         <v>277</v>
       </c>
@@ -19588,7 +19585,7 @@
         <v>0.28873287738484599</v>
       </c>
     </row>
-    <row r="269" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A269" s="1" t="s">
         <v>278</v>
       </c>
@@ -19599,7 +19596,7 @@
         <v>0.28985427653153101</v>
       </c>
     </row>
-    <row r="270" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A270" s="1" t="s">
         <v>279</v>
       </c>
@@ -19610,7 +19607,7 @@
         <v>0.29473582812057803</v>
       </c>
     </row>
-    <row r="271" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A271" s="1" t="s">
         <v>280</v>
       </c>
@@ -19621,7 +19618,7 @@
         <v>0.29630016894823502</v>
       </c>
     </row>
-    <row r="272" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A272" s="1" t="s">
         <v>281</v>
       </c>
@@ -19632,7 +19629,7 @@
         <v>0.290375757335809</v>
       </c>
     </row>
-    <row r="273" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A273" s="1" t="s">
         <v>282</v>
       </c>
@@ -19643,7 +19640,7 @@
         <v>0.29184259037329402</v>
       </c>
     </row>
-    <row r="274" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A274" s="1" t="s">
         <v>283</v>
       </c>
@@ -19654,7 +19651,7 @@
         <v>0.29495272762742802</v>
       </c>
     </row>
-    <row r="275" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A275" s="1" t="s">
         <v>284</v>
       </c>
@@ -19665,7 +19662,7 @@
         <v>0.29546767207366198</v>
       </c>
     </row>
-    <row r="276" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A276" s="1" t="s">
         <v>285</v>
       </c>
@@ -19676,7 +19673,7 @@
         <v>0.29613521382059799</v>
       </c>
     </row>
-    <row r="277" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A277" s="1" t="s">
         <v>286</v>
       </c>
@@ -19687,7 +19684,7 @@
         <v>0.29582825670155199</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A278" s="1" t="s">
         <v>287</v>
       </c>
@@ -19698,7 +19695,7 @@
         <v>0.29449530569974303</v>
       </c>
     </row>
-    <row r="279" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A279" s="1" t="s">
         <v>288</v>
       </c>
@@ -19709,7 +19706,7 @@
         <v>0.29806425275037302</v>
       </c>
     </row>
-    <row r="280" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A280" s="1" t="s">
         <v>289</v>
       </c>
@@ -19720,7 +19717,7 @@
         <v>0.29361605170472399</v>
       </c>
     </row>
-    <row r="281" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A281" s="1" t="s">
         <v>290</v>
       </c>
@@ -19731,7 +19728,7 @@
         <v>0.29750345759486801</v>
       </c>
     </row>
-    <row r="282" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A282" s="1" t="s">
         <v>291</v>
       </c>
@@ -19742,7 +19739,7 @@
         <v>0.29221770492358401</v>
       </c>
     </row>
-    <row r="283" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A283" s="1" t="s">
         <v>292</v>
       </c>
@@ -19753,7 +19750,7 @@
         <v>0.29462962623990302</v>
       </c>
     </row>
-    <row r="284" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A284" s="1" t="s">
         <v>293</v>
       </c>
@@ -19764,7 +19761,7 @@
         <v>0.29592312403825599</v>
       </c>
     </row>
-    <row r="285" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A285" s="1" t="s">
         <v>294</v>
       </c>
@@ -19775,7 +19772,7 @@
         <v>0.29448024773360298</v>
       </c>
     </row>
-    <row r="286" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A286" s="1" t="s">
         <v>295</v>
       </c>
@@ -19786,7 +19783,7 @@
         <v>0.29587930445673999</v>
       </c>
     </row>
-    <row r="287" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A287" s="1" t="s">
         <v>296</v>
       </c>
@@ -19797,7 +19794,7 @@
         <v>0.28842517989208999</v>
       </c>
     </row>
-    <row r="288" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A288" s="1" t="s">
         <v>297</v>
       </c>
@@ -19808,7 +19805,7 @@
         <v>0.29360342062414901</v>
       </c>
     </row>
-    <row r="289" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A289" s="1" t="s">
         <v>298</v>
       </c>
@@ -19819,7 +19816,7 @@
         <v>0.28921987206488498</v>
       </c>
     </row>
-    <row r="290" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A290" s="1" t="s">
         <v>299</v>
       </c>
@@ -19830,7 +19827,7 @@
         <v>0.29134851176696303</v>
       </c>
     </row>
-    <row r="291" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A291" s="1" t="s">
         <v>300</v>
       </c>
@@ -19841,7 +19838,7 @@
         <v>0.29264779346075898</v>
       </c>
     </row>
-    <row r="292" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A292" s="1" t="s">
         <v>301</v>
       </c>
@@ -19852,7 +19849,7 @@
         <v>0.28825504808202801</v>
       </c>
     </row>
-    <row r="293" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A293" s="1" t="s">
         <v>302</v>
       </c>
@@ -19863,7 +19860,7 @@
         <v>0.29422715038680303</v>
       </c>
     </row>
-    <row r="294" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A294" s="1" t="s">
         <v>303</v>
       </c>
@@ -19874,7 +19871,7 @@
         <v>0.295993095562951</v>
       </c>
     </row>
-    <row r="295" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A295" s="1" t="s">
         <v>304</v>
       </c>
@@ -19885,7 +19882,7 @@
         <v>0.291643296428021</v>
       </c>
     </row>
-    <row r="296" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A296" s="1" t="s">
         <v>305</v>
       </c>
@@ -19896,7 +19893,7 @@
         <v>0.29408431924388001</v>
       </c>
     </row>
-    <row r="297" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:3" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A297" s="1" t="s">
         <v>306</v>
       </c>
@@ -19917,13 +19914,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D318508-EB39-4B19-9441-3235666F09D0}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.41796875" customWidth="1"/>
+    <col min="2" max="2" width="11.578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>208</v>
       </c>
@@ -19976,7 +19973,7 @@
         <v>4.8722013994164027E-4</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>209</v>
       </c>
@@ -20029,7 +20026,7 @@
         <v>0.16607519486925235</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>207</v>
       </c>
@@ -20070,7 +20067,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>1</v>
       </c>
@@ -20111,7 +20108,7 @@
         <v>0.29193451692567801</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>2</v>
       </c>
@@ -20152,7 +20149,7 @@
         <v>0.28873287738484599</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>3</v>
       </c>
@@ -20193,7 +20190,7 @@
         <v>0.28985427653153101</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>4</v>
       </c>
@@ -20234,7 +20231,7 @@
         <v>0.29473582812057803</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>5</v>
       </c>
@@ -20275,7 +20272,7 @@
         <v>0.29630016894823502</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>6</v>
       </c>
@@ -20313,7 +20310,7 @@
         <v>0.290375757335809</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>7</v>
       </c>
@@ -20351,7 +20348,7 @@
         <v>0.29184259037329402</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>8</v>
       </c>
@@ -20389,7 +20386,7 @@
         <v>0.29495272762742802</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>9</v>
       </c>
@@ -20427,7 +20424,7 @@
         <v>0.29546767207366198</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>10</v>
       </c>
@@ -20465,7 +20462,7 @@
         <v>0.29613521382059799</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>11</v>
       </c>
@@ -20503,7 +20500,7 @@
         <v>0.29582825670155199</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>12</v>
       </c>
@@ -20541,7 +20538,7 @@
         <v>0.29449530569974303</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>13</v>
       </c>
@@ -20579,7 +20576,7 @@
         <v>0.29806425275037302</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>14</v>
       </c>
@@ -20617,7 +20614,7 @@
         <v>0.29361605170472399</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>15</v>
       </c>
@@ -20655,7 +20652,7 @@
         <v>0.29750345759486801</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>16</v>
       </c>
@@ -20690,7 +20687,7 @@
         <v>0.29221770492358401</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>17</v>
       </c>
@@ -20722,7 +20719,7 @@
         <v>0.29462962623990302</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>18</v>
       </c>
@@ -20754,7 +20751,7 @@
         <v>0.29592312403825599</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>19</v>
       </c>
@@ -20786,7 +20783,7 @@
         <v>0.29448024773360298</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
         <v>20</v>
       </c>
@@ -20815,7 +20812,7 @@
         <v>0.29587930445673999</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
         <v>21</v>
       </c>
@@ -20841,7 +20838,7 @@
         <v>0.28842517989208999</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
         <v>22</v>
       </c>
@@ -20867,7 +20864,7 @@
         <v>0.29360342062414901</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A26">
         <v>23</v>
       </c>
@@ -20893,7 +20890,7 @@
         <v>0.28921987206488498</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A27">
         <v>24</v>
       </c>
@@ -20916,7 +20913,7 @@
         <v>0.29134851176696303</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A28">
         <v>25</v>
       </c>
@@ -20939,7 +20936,7 @@
         <v>0.29264779346075898</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A29">
         <v>26</v>
       </c>
@@ -20962,7 +20959,7 @@
         <v>0.28825504808202801</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A30">
         <v>27</v>
       </c>
@@ -20985,7 +20982,7 @@
         <v>0.29422715038680303</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A31">
         <v>28</v>
       </c>
@@ -21008,7 +21005,7 @@
         <v>0.295993095562951</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A32">
         <v>29</v>
       </c>
@@ -21028,7 +21025,7 @@
         <v>0.291643296428021</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A33">
         <v>30</v>
       </c>
@@ -21048,7 +21045,7 @@
         <v>0.29408431924388001</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A34">
         <v>31</v>
       </c>
@@ -21068,7 +21065,7 @@
         <v>0.29215304331091801</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A35">
         <v>32</v>
       </c>
@@ -21079,7 +21076,7 @@
         <v>0.22249606599096799</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A36">
         <v>33</v>
       </c>
@@ -21087,7 +21084,7 @@
         <v>0.22770140189949001</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A37">
         <v>34</v>
       </c>
@@ -21095,7 +21092,7 @@
         <v>0.22467693879523801</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A38">
         <v>35</v>
       </c>
@@ -21103,7 +21100,7 @@
         <v>0.22590951148508701</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A39">
         <v>36</v>
       </c>
@@ -21121,12 +21118,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A5AE877-64C3-4028-8147-765389663D58}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.68359375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>208</v>
       </c>
@@ -21179,7 +21176,7 @@
         <v>1.5436675245504185E-2</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>209</v>
       </c>
@@ -21232,7 +21229,7 @@
         <v>8.55645429483185E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>207</v>
       </c>
@@ -21273,7 +21270,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>1</v>
       </c>
@@ -21314,7 +21311,7 @@
         <v>17.825013007136501</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>2</v>
       </c>
@@ -21355,7 +21352,7 @@
         <v>17.9319730766783</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>3</v>
       </c>
@@ -21396,7 +21393,7 @@
         <v>18.039044650769</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>4</v>
       </c>
@@ -21437,7 +21434,7 @@
         <v>18.0604756933053</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>5</v>
       </c>
@@ -21478,7 +21475,7 @@
         <v>17.9979172106978</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>6</v>
       </c>
@@ -21516,7 +21513,7 @@
         <v>17.998827423434999</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>7</v>
       </c>
@@ -21554,7 +21551,7 @@
         <v>18.041509768701101</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>8</v>
       </c>
@@ -21592,7 +21589,7 @@
         <v>18.113057907959</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>9</v>
       </c>
@@ -21630,7 +21627,7 @@
         <v>18.000340035364701</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>10</v>
       </c>
@@ -21668,7 +21665,7 @@
         <v>18.056008326627001</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>11</v>
       </c>
@@ -21706,7 +21703,7 @@
         <v>18.143480906181601</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>12</v>
       </c>
@@ -21744,7 +21741,7 @@
         <v>18.0505063076521</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>13</v>
       </c>
@@ -21782,7 +21779,7 @@
         <v>17.975837914720699</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>14</v>
       </c>
@@ -21820,7 +21817,7 @@
         <v>17.958408612980101</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>15</v>
       </c>
@@ -21858,7 +21855,7 @@
         <v>18.089794941394199</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>16</v>
       </c>
@@ -21893,7 +21890,7 @@
         <v>18.011107051113001</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>17</v>
       </c>
@@ -21925,7 +21922,7 @@
         <v>18.059805482066999</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>18</v>
       </c>
@@ -21957,7 +21954,7 @@
         <v>17.9483749982906</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>19</v>
       </c>
@@ -21989,7 +21986,7 @@
         <v>17.986594818813899</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
         <v>20</v>
       </c>
@@ -22018,7 +22015,7 @@
         <v>18.0136321630971</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
         <v>21</v>
       </c>
@@ -22044,7 +22041,7 @@
         <v>18.175378572568899</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
         <v>22</v>
       </c>
@@ -22070,7 +22067,7 @@
         <v>18.118575471661899</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A26">
         <v>23</v>
       </c>
@@ -22096,7 +22093,7 @@
         <v>17.929983986435602</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A27">
         <v>24</v>
       </c>
@@ -22119,7 +22116,7 @@
         <v>18.106604307150199</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A28">
         <v>25</v>
       </c>
@@ -22142,7 +22139,7 @@
         <v>17.996855885347902</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A29">
         <v>26</v>
       </c>
@@ -22165,7 +22162,7 @@
         <v>18.121396667491499</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A30">
         <v>27</v>
       </c>
@@ -22188,7 +22185,7 @@
         <v>18.094216738234799</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A31">
         <v>28</v>
       </c>
@@ -22211,7 +22208,7 @@
         <v>18.1174045096291</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A32">
         <v>29</v>
       </c>
@@ -22231,7 +22228,7 @@
         <v>17.975345051957699</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A33">
         <v>30</v>
       </c>
@@ -22251,7 +22248,7 @@
         <v>18.0641154539816</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A34">
         <v>31</v>
       </c>
@@ -22271,7 +22268,7 @@
         <v>18.268545430641002</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A35">
         <v>32</v>
       </c>
@@ -22282,7 +22279,7 @@
         <v>13.9597270287277</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A36">
         <v>33</v>
       </c>
@@ -22290,7 +22287,7 @@
         <v>13.946102058433601</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A37">
         <v>34</v>
       </c>
@@ -22298,7 +22295,7 @@
         <v>13.9823014618208</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A38">
         <v>35</v>
       </c>
@@ -22306,7 +22303,7 @@
         <v>13.749906400784599</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A39">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
Try Rerun again with gamma not changing
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=3.xlsx
+++ b/Fit Results/AllFitsF1=3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B52CCC-E55F-4EDB-853A-87FBB98AAEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5A71CF-ADCE-4411-8600-F7F5E0BA409C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Together" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Working on overall lin fit
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=3.xlsx
+++ b/Fit Results/AllFitsF1=3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\Fit Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F309F427-6C09-4F12-81A5-00FE6CDB3860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C37905-4062-4D15-ABB2-40EBDEB099B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="5280" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Together" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -3260,7 +3263,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3268,6 +3270,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -5985,7 +5988,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -5993,6 +5995,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9168,7 +9171,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9176,6 +9178,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9669,7 +9672,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9677,6 +9679,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12237,7 +12240,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12245,6 +12247,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12738,7 +12741,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12746,6 +12748,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16156,16 +16159,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>467265</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>44928</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>242618</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>494220</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>152760</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>284309</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>539151</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>158507</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -16611,12 +16614,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R297"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="6" width="16.1796875" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -16634,7 +16637,7 @@
       </c>
       <c r="R1" s="1"/>
     </row>
-    <row r="2" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -16660,7 +16663,7 @@
         <v>4.2703475132141157E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -16682,7 +16685,7 @@
         <v>0.18809412531311234</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -16694,7 +16697,7 @@
       </c>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -16716,7 +16719,7 @@
         <v>0.22378459935658199</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -16738,7 +16741,7 @@
         <v>0.228434718604688</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -16760,7 +16763,7 @@
         <v>0.221372998488612</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
@@ -16782,7 +16785,7 @@
         <v>0.225975457594905</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
@@ -16804,7 +16807,7 @@
         <v>0.225216837741747</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>309</v>
       </c>
@@ -16826,7 +16829,7 @@
         <v>0.229746279532067</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>310</v>
       </c>
@@ -16848,7 +16851,7 @@
         <v>0.22722518963626401</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -16870,7 +16873,7 @@
         <v>0.222965184868961</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>311</v>
       </c>
@@ -16892,7 +16895,7 @@
         <v>0.22898718060617901</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -16903,7 +16906,7 @@
         <v>0.13498234565869699</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -16914,7 +16917,7 @@
         <v>0.13854180631109</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -16925,7 +16928,7 @@
         <v>0.13743837454275501</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -16936,7 +16939,7 @@
         <v>0.13738267695902801</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
@@ -16947,7 +16950,7 @@
         <v>0.14159428045373601</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
@@ -16958,7 +16961,7 @@
         <v>0.14232784705226301</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>13</v>
       </c>
@@ -16969,7 +16972,7 @@
         <v>0.14391242117178599</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
@@ -16980,7 +16983,7 @@
         <v>0.13920272125085101</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>15</v>
       </c>
@@ -16991,7 +16994,7 @@
         <v>0.14459533841685501</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>312</v>
       </c>
@@ -17002,7 +17005,7 @@
         <v>0.13915991329959099</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>16</v>
       </c>
@@ -17013,7 +17016,7 @@
         <v>0.144975058104169</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
@@ -17024,7 +17027,7 @@
         <v>0.14496624110967199</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>18</v>
       </c>
@@ -17035,7 +17038,7 @@
         <v>0.14341121488491801</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>19</v>
       </c>
@@ -17046,7 +17049,7 @@
         <v>0.14388771373763901</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>20</v>
       </c>
@@ -17057,7 +17060,7 @@
         <v>0.14091026017191899</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>313</v>
       </c>
@@ -17068,7 +17071,7 @@
         <v>0.13928443937518301</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>21</v>
       </c>
@@ -17079,7 +17082,7 @@
         <v>0.14449758570660601</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>314</v>
       </c>
@@ -17090,7 +17093,7 @@
         <v>0.14272080636913501</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>315</v>
       </c>
@@ -17101,7 +17104,7 @@
         <v>0.14380448214622399</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>22</v>
       </c>
@@ -17112,7 +17115,7 @@
         <v>0.13910873933717599</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>28</v>
       </c>
@@ -17123,7 +17126,7 @@
         <v>0.117218052017694</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>29</v>
       </c>
@@ -17134,7 +17137,7 @@
         <v>0.116738218899043</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>30</v>
       </c>
@@ -17145,7 +17148,7 @@
         <v>0.116641895814922</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>31</v>
       </c>
@@ -17156,7 +17159,7 @@
         <v>0.117986722306339</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>32</v>
       </c>
@@ -17167,7 +17170,7 @@
         <v>0.116363944216263</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>33</v>
       </c>
@@ -17178,7 +17181,7 @@
         <v>0.117960737624138</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>34</v>
       </c>
@@ -17189,7 +17192,7 @@
         <v>0.11777189549636199</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>35</v>
       </c>
@@ -17200,7 +17203,7 @@
         <v>0.118362346500101</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>36</v>
       </c>
@@ -17211,7 +17214,7 @@
         <v>0.11875028071223</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>37</v>
       </c>
@@ -17222,7 +17225,7 @@
         <v>0.118209453954305</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>38</v>
       </c>
@@ -17233,7 +17236,7 @@
         <v>0.116577694816434</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>39</v>
       </c>
@@ -17244,7 +17247,7 @@
         <v>0.117670638852321</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>40</v>
       </c>
@@ -17255,7 +17258,7 @@
         <v>0.118098845799444</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>41</v>
       </c>
@@ -17266,7 +17269,7 @@
         <v>0.11655919684067299</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>42</v>
       </c>
@@ -17277,7 +17280,7 @@
         <v>0.118487075826876</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>43</v>
       </c>
@@ -17288,7 +17291,7 @@
         <v>0.117049111989703</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>44</v>
       </c>
@@ -17299,7 +17302,7 @@
         <v>0.116964493443121</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>45</v>
       </c>
@@ -17310,7 +17313,7 @@
         <v>0.1174932059815</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>46</v>
       </c>
@@ -17321,7 +17324,7 @@
         <v>0.118724780988732</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>47</v>
       </c>
@@ -17332,7 +17335,7 @@
         <v>0.11857414162119</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>48</v>
       </c>
@@ -17343,7 +17346,7 @@
         <v>0.116857985488521</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>49</v>
       </c>
@@ -17354,7 +17357,7 @@
         <v>0.117839930521939</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>50</v>
       </c>
@@ -17365,7 +17368,7 @@
         <v>0.116123290748398</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>51</v>
       </c>
@@ -17376,7 +17379,7 @@
         <v>0.116339626646247</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>52</v>
       </c>
@@ -17387,7 +17390,7 @@
         <v>0.118521454357363</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>53</v>
       </c>
@@ -17398,7 +17401,7 @@
         <v>0.117743388207075</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>54</v>
       </c>
@@ -17409,7 +17412,7 @@
         <v>0.116823099810358</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>55</v>
       </c>
@@ -17420,7 +17423,7 @@
         <v>0.118509294607666</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>56</v>
       </c>
@@ -17431,7 +17434,7 @@
         <v>0.118631007440724</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>57</v>
       </c>
@@ -17442,7 +17445,7 @@
         <v>0.117484320873481</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>58</v>
       </c>
@@ -17453,7 +17456,7 @@
         <v>0.118251546607688</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>59</v>
       </c>
@@ -17464,7 +17467,7 @@
         <v>0.118181098472526</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>60</v>
       </c>
@@ -17475,7 +17478,7 @@
         <v>8.9287039240001795E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>61</v>
       </c>
@@ -17486,7 +17489,7 @@
         <v>8.9953273584561996E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>62</v>
       </c>
@@ -17497,7 +17500,7 @@
         <v>9.1230909809772498E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>63</v>
       </c>
@@ -17508,7 +17511,7 @@
         <v>9.0037965159722497E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>64</v>
       </c>
@@ -17519,7 +17522,7 @@
         <v>9.2063662732121604E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>65</v>
       </c>
@@ -17530,7 +17533,7 @@
         <v>9.0566169869859395E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>66</v>
       </c>
@@ -17541,7 +17544,7 @@
         <v>9.1281359996997199E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>67</v>
       </c>
@@ -17552,7 +17555,7 @@
         <v>9.0246189977935598E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>68</v>
       </c>
@@ -17563,7 +17566,7 @@
         <v>8.7987770056780296E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>69</v>
       </c>
@@ -17574,7 +17577,7 @@
         <v>9.1038024594974204E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>70</v>
       </c>
@@ -17585,7 +17588,7 @@
         <v>9.0356969610468907E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>71</v>
       </c>
@@ -17596,7 +17599,7 @@
         <v>8.9055177802521202E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>72</v>
       </c>
@@ -17607,7 +17610,7 @@
         <v>9.0556231765949805E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>73</v>
       </c>
@@ -17618,7 +17621,7 @@
         <v>9.1259865204828206E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>74</v>
       </c>
@@ -17629,7 +17632,7 @@
         <v>8.8371089308141498E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>75</v>
       </c>
@@ -17640,7 +17643,7 @@
         <v>8.9886315679026302E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>76</v>
       </c>
@@ -17651,7 +17654,7 @@
         <v>0.22378459935658199</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>77</v>
       </c>
@@ -17662,7 +17665,7 @@
         <v>0.228434718604688</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>78</v>
       </c>
@@ -17673,7 +17676,7 @@
         <v>0.221372998488612</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>79</v>
       </c>
@@ -17684,7 +17687,7 @@
         <v>0.225975457594905</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>80</v>
       </c>
@@ -17695,7 +17698,7 @@
         <v>0.225216837741747</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>81</v>
       </c>
@@ -17706,7 +17709,7 @@
         <v>0.229746279532067</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>82</v>
       </c>
@@ -17717,7 +17720,7 @@
         <v>0.22722518963626401</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>83</v>
       </c>
@@ -17728,7 +17731,7 @@
         <v>0.222965184868961</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>84</v>
       </c>
@@ -17739,7 +17742,7 @@
         <v>0.22898718060617901</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>85</v>
       </c>
@@ -17750,7 +17753,7 @@
         <v>0.22580668748875701</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>86</v>
       </c>
@@ -17761,7 +17764,7 @@
         <v>0.231594890582631</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>87</v>
       </c>
@@ -17772,7 +17775,7 @@
         <v>0.224583618990919</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>88</v>
       </c>
@@ -17783,7 +17786,7 @@
         <v>0.23249128317182099</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>89</v>
       </c>
@@ -17794,7 +17797,7 @@
         <v>0.23073510515949899</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>90</v>
       </c>
@@ -17805,7 +17808,7 @@
         <v>0.229179326874075</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>91</v>
       </c>
@@ -17816,7 +17819,7 @@
         <v>0.226024665246639</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>92</v>
       </c>
@@ -17827,7 +17830,7 @@
         <v>0.22988414195496401</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>93</v>
       </c>
@@ -17838,7 +17841,7 @@
         <v>0.22795719930278499</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>94</v>
       </c>
@@ -17849,7 +17852,7 @@
         <v>0.227267035209756</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>95</v>
       </c>
@@ -17860,7 +17863,7 @@
         <v>0.22728875634974799</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>96</v>
       </c>
@@ -17871,7 +17874,7 @@
         <v>0.22819660608103401</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>97</v>
       </c>
@@ -17882,7 +17885,7 @@
         <v>0.22449918198189101</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>98</v>
       </c>
@@ -17893,7 +17896,7 @@
         <v>0.22352994908158599</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>99</v>
       </c>
@@ -17904,7 +17907,7 @@
         <v>0.22753327784977401</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>100</v>
       </c>
@@ -17915,7 +17918,7 @@
         <v>0.22784419865740199</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>101</v>
       </c>
@@ -17926,7 +17929,7 @@
         <v>0.225433003733543</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>102</v>
       </c>
@@ -17937,7 +17940,7 @@
         <v>0.22712348211729699</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>103</v>
       </c>
@@ -17948,7 +17951,7 @@
         <v>0.22894109101944199</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>104</v>
       </c>
@@ -17959,7 +17962,7 @@
         <v>0.23027592968354901</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>105</v>
       </c>
@@ -17970,7 +17973,7 @@
         <v>0.22733899516780401</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>106</v>
       </c>
@@ -17981,7 +17984,7 @@
         <v>0.22718964047891599</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>107</v>
       </c>
@@ -17992,7 +17995,7 @@
         <v>0.22249606599096799</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>108</v>
       </c>
@@ -18003,7 +18006,7 @@
         <v>0.22770140189949001</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>109</v>
       </c>
@@ -18014,7 +18017,7 @@
         <v>0.22467693879523801</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>110</v>
       </c>
@@ -18025,7 +18028,7 @@
         <v>0.22590951148508701</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>111</v>
       </c>
@@ -18036,7 +18039,7 @@
         <v>0.22795873224990801</v>
       </c>
     </row>
-    <row r="118" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>112</v>
       </c>
@@ -18047,7 +18050,7 @@
         <v>0.26064960163891099</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>113</v>
       </c>
@@ -18058,7 +18061,7 @@
         <v>0.25338188968269398</v>
       </c>
     </row>
-    <row r="120" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>114</v>
       </c>
@@ -18069,7 +18072,7 @@
         <v>0.25038094455952498</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>115</v>
       </c>
@@ -18080,7 +18083,7 @@
         <v>0.256215228918099</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>116</v>
       </c>
@@ -18091,7 +18094,7 @@
         <v>0.25483329669185101</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>117</v>
       </c>
@@ -18102,7 +18105,7 @@
         <v>0.25854387484878599</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>118</v>
       </c>
@@ -18113,7 +18116,7 @@
         <v>0.25519336396030601</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>119</v>
       </c>
@@ -18124,7 +18127,7 @@
         <v>0.25663303680948102</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>120</v>
       </c>
@@ -18135,7 +18138,7 @@
         <v>0.25601459599486398</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>121</v>
       </c>
@@ -18146,7 +18149,7 @@
         <v>0.25648553124648299</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>122</v>
       </c>
@@ -18157,7 +18160,7 @@
         <v>0.25339182435774998</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>123</v>
       </c>
@@ -18168,7 +18171,7 @@
         <v>0.26261256236820102</v>
       </c>
     </row>
-    <row r="130" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>124</v>
       </c>
@@ -18179,7 +18182,7 @@
         <v>0.25914013258546797</v>
       </c>
     </row>
-    <row r="131" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>125</v>
       </c>
@@ -18190,7 +18193,7 @@
         <v>0.25187380012057398</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>126</v>
       </c>
@@ -18201,7 +18204,7 @@
         <v>0.25861462842520899</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>127</v>
       </c>
@@ -18212,7 +18215,7 @@
         <v>0.26412000142144099</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>128</v>
       </c>
@@ -18223,7 +18226,7 @@
         <v>0.25505739125523702</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>129</v>
       </c>
@@ -18234,7 +18237,7 @@
         <v>0.25268334549192301</v>
       </c>
     </row>
-    <row r="136" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>130</v>
       </c>
@@ -18245,7 +18248,7 @@
         <v>0.254203134019032</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>131</v>
       </c>
@@ -18256,7 +18259,7 @@
         <v>0.25355249186689299</v>
       </c>
     </row>
-    <row r="138" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>132</v>
       </c>
@@ -18267,7 +18270,7 @@
         <v>0.258640908855092</v>
       </c>
     </row>
-    <row r="139" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>133</v>
       </c>
@@ -18278,7 +18281,7 @@
         <v>0.25176887581155899</v>
       </c>
     </row>
-    <row r="140" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>134</v>
       </c>
@@ -18289,7 +18292,7 @@
         <v>0.25436276153236997</v>
       </c>
     </row>
-    <row r="141" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>135</v>
       </c>
@@ -18300,7 +18303,7 @@
         <v>0.25848980394328103</v>
       </c>
     </row>
-    <row r="142" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>136</v>
       </c>
@@ -18311,7 +18314,7 @@
         <v>0.25493042534243598</v>
       </c>
     </row>
-    <row r="143" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>137</v>
       </c>
@@ -18322,7 +18325,7 @@
         <v>0.25702073078272197</v>
       </c>
     </row>
-    <row r="144" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>138</v>
       </c>
@@ -18333,7 +18336,7 @@
         <v>0.25281370286486299</v>
       </c>
     </row>
-    <row r="145" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>139</v>
       </c>
@@ -18344,7 +18347,7 @@
         <v>0.25787828139437702</v>
       </c>
     </row>
-    <row r="146" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>140</v>
       </c>
@@ -18355,7 +18358,7 @@
         <v>0.255030114263046</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>141</v>
       </c>
@@ -18366,7 +18369,7 @@
         <v>0.25326708245889501</v>
       </c>
     </row>
-    <row r="148" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>142</v>
       </c>
@@ -18377,7 +18380,7 @@
         <v>0.25901851572451601</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>143</v>
       </c>
@@ -18388,7 +18391,7 @@
         <v>0.25402214979933802</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>144</v>
       </c>
@@ -18399,7 +18402,7 @@
         <v>0.25207440807669201</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>145</v>
       </c>
@@ -18410,7 +18413,7 @@
         <v>0.25648835225167999</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>146</v>
       </c>
@@ -18421,7 +18424,7 @@
         <v>0.25619702232418301</v>
       </c>
     </row>
-    <row r="153" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>147</v>
       </c>
@@ -18432,7 +18435,7 @@
         <v>0.256904989972564</v>
       </c>
     </row>
-    <row r="154" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>148</v>
       </c>
@@ -18443,7 +18446,7 @@
         <v>0.25656545981822299</v>
       </c>
     </row>
-    <row r="155" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>149</v>
       </c>
@@ -18454,7 +18457,7 @@
         <v>0.25471437628790899</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>150</v>
       </c>
@@ -18465,7 +18468,7 @@
         <v>0.25564492601438199</v>
       </c>
     </row>
-    <row r="157" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>151</v>
       </c>
@@ -18476,7 +18479,7 @@
         <v>0.26266359379455601</v>
       </c>
     </row>
-    <row r="158" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>152</v>
       </c>
@@ -18487,7 +18490,7 @@
         <v>0.25914186884267898</v>
       </c>
     </row>
-    <row r="159" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>153</v>
       </c>
@@ -18498,7 +18501,7 @@
         <v>0.25621155685651098</v>
       </c>
     </row>
-    <row r="160" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>154</v>
       </c>
@@ -18509,7 +18512,7 @@
         <v>0.25866494788723898</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>155</v>
       </c>
@@ -18520,7 +18523,7 @@
         <v>0.25801756322347102</v>
       </c>
     </row>
-    <row r="162" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>156</v>
       </c>
@@ -18531,7 +18534,7 @@
         <v>0.25944545650678502</v>
       </c>
     </row>
-    <row r="163" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>157</v>
       </c>
@@ -18542,7 +18545,7 @@
         <v>0.25336488450504602</v>
       </c>
     </row>
-    <row r="164" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>158</v>
       </c>
@@ -18553,7 +18556,7 @@
         <v>0.261553420142073</v>
       </c>
     </row>
-    <row r="165" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>159</v>
       </c>
@@ -18564,7 +18567,7 @@
         <v>0.26019522603942802</v>
       </c>
     </row>
-    <row r="166" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>160</v>
       </c>
@@ -18575,7 +18578,7 @@
         <v>0.25868729407005198</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>161</v>
       </c>
@@ -18586,7 +18589,7 @@
         <v>0.25516460879894798</v>
       </c>
     </row>
-    <row r="168" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>162</v>
       </c>
@@ -18597,7 +18600,7 @@
         <v>0.25295075090609098</v>
       </c>
     </row>
-    <row r="169" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>163</v>
       </c>
@@ -18608,7 +18611,7 @@
         <v>0.256452611497334</v>
       </c>
     </row>
-    <row r="170" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>164</v>
       </c>
@@ -18619,7 +18622,7 @@
         <v>0.25868777299010298</v>
       </c>
     </row>
-    <row r="171" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>165</v>
       </c>
@@ -18630,7 +18633,7 @@
         <v>0.2539674766801</v>
       </c>
     </row>
-    <row r="172" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>166</v>
       </c>
@@ -18641,7 +18644,7 @@
         <v>0.17294771128421699</v>
       </c>
     </row>
-    <row r="173" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>167</v>
       </c>
@@ -18652,7 +18655,7 @@
         <v>0.175665485735155</v>
       </c>
     </row>
-    <row r="174" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>168</v>
       </c>
@@ -18663,7 +18666,7 @@
         <v>0.17382778027635701</v>
       </c>
     </row>
-    <row r="175" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>169</v>
       </c>
@@ -18674,7 +18677,7 @@
         <v>0.17455983570099701</v>
       </c>
     </row>
-    <row r="176" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>170</v>
       </c>
@@ -18685,7 +18688,7 @@
         <v>0.17664296551393399</v>
       </c>
     </row>
-    <row r="177" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>171</v>
       </c>
@@ -18696,7 +18699,7 @@
         <v>0.17708531560420199</v>
       </c>
     </row>
-    <row r="178" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>172</v>
       </c>
@@ -18707,7 +18710,7 @@
         <v>0.17557573140333699</v>
       </c>
     </row>
-    <row r="179" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>173</v>
       </c>
@@ -18718,7 +18721,7 @@
         <v>0.173457649972002</v>
       </c>
     </row>
-    <row r="180" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>174</v>
       </c>
@@ -18729,7 +18732,7 @@
         <v>0.17535865105134299</v>
       </c>
     </row>
-    <row r="181" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>175</v>
       </c>
@@ -18740,7 +18743,7 @@
         <v>0.175039518424147</v>
       </c>
     </row>
-    <row r="182" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>176</v>
       </c>
@@ -18751,7 +18754,7 @@
         <v>0.17459939950666101</v>
       </c>
     </row>
-    <row r="183" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>177</v>
       </c>
@@ -18762,7 +18765,7 @@
         <v>0.17177387798819599</v>
       </c>
     </row>
-    <row r="184" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>178</v>
       </c>
@@ -18773,7 +18776,7 @@
         <v>0.172049396498035</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>179</v>
       </c>
@@ -18784,7 +18787,7 @@
         <v>0.17416028353340501</v>
       </c>
     </row>
-    <row r="186" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>180</v>
       </c>
@@ -18795,7 +18798,7 @@
         <v>0.17432866559164001</v>
       </c>
     </row>
-    <row r="187" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>181</v>
       </c>
@@ -18806,7 +18809,7 @@
         <v>0.17371638201273101</v>
       </c>
     </row>
-    <row r="188" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>182</v>
       </c>
@@ -18817,7 +18820,7 @@
         <v>0.17123203171632401</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>183</v>
       </c>
@@ -18828,7 +18831,7 @@
         <v>0.17318569822136001</v>
       </c>
     </row>
-    <row r="190" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>184</v>
       </c>
@@ -18839,7 +18842,7 @@
         <v>0.17669669700448201</v>
       </c>
     </row>
-    <row r="191" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>185</v>
       </c>
@@ -18850,7 +18853,7 @@
         <v>0.17723933870696301</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>186</v>
       </c>
@@ -18861,7 +18864,7 @@
         <v>0.17063092731327101</v>
       </c>
     </row>
-    <row r="193" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>187</v>
       </c>
@@ -18872,7 +18875,7 @@
         <v>0.17490193092626999</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>188</v>
       </c>
@@ -18883,7 +18886,7 @@
         <v>0.17702310390171999</v>
       </c>
     </row>
-    <row r="195" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>189</v>
       </c>
@@ -18894,7 +18897,7 @@
         <v>0.171948853936535</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>190</v>
       </c>
@@ -18905,7 +18908,7 @@
         <v>0.17411860264206899</v>
       </c>
     </row>
-    <row r="197" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>191</v>
       </c>
@@ -18916,7 +18919,7 @@
         <v>0.175935205113702</v>
       </c>
     </row>
-    <row r="198" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>192</v>
       </c>
@@ -18927,7 +18930,7 @@
         <v>0.17427622300988699</v>
       </c>
     </row>
-    <row r="199" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>193</v>
       </c>
@@ -18938,7 +18941,7 @@
         <v>0.17224969239811899</v>
       </c>
     </row>
-    <row r="200" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>194</v>
       </c>
@@ -18949,7 +18952,7 @@
         <v>0.17435257559575301</v>
       </c>
     </row>
-    <row r="201" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>195</v>
       </c>
@@ -18960,7 +18963,7 @@
         <v>0.171222354567128</v>
       </c>
     </row>
-    <row r="202" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>196</v>
       </c>
@@ -18971,7 +18974,7 @@
         <v>0.17230494746765301</v>
       </c>
     </row>
-    <row r="203" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>197</v>
       </c>
@@ -18982,7 +18985,7 @@
         <v>0.17976030708667101</v>
       </c>
     </row>
-    <row r="204" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>198</v>
       </c>
@@ -18993,7 +18996,7 @@
         <v>0.174433801903358</v>
       </c>
     </row>
-    <row r="205" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>199</v>
       </c>
@@ -19004,7 +19007,7 @@
         <v>0.17714435708530099</v>
       </c>
     </row>
-    <row r="206" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>200</v>
       </c>
@@ -19015,7 +19018,7 @@
         <v>0.17086804073973499</v>
       </c>
     </row>
-    <row r="207" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>201</v>
       </c>
@@ -19026,7 +19029,7 @@
         <v>0.171697248433512</v>
       </c>
     </row>
-    <row r="208" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>202</v>
       </c>
@@ -19037,7 +19040,7 @@
         <v>0.17443666559002999</v>
       </c>
     </row>
-    <row r="209" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>203</v>
       </c>
@@ -19048,7 +19051,7 @@
         <v>0.17690051952166999</v>
       </c>
     </row>
-    <row r="210" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>204</v>
       </c>
@@ -19059,19 +19062,19 @@
         <v>0.17654554655181801</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
       <c r="C211" s="1"/>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
     </row>
-    <row r="214" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>245</v>
       </c>
@@ -19082,7 +19085,7 @@
         <v>0.21689563024651701</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>246</v>
       </c>
@@ -19093,7 +19096,7 @@
         <v>0.21250705902688999</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>247</v>
       </c>
@@ -19104,7 +19107,7 @@
         <v>0.21268324019514501</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>248</v>
       </c>
@@ -19115,7 +19118,7 @@
         <v>0.21049345542616399</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>249</v>
       </c>
@@ -19126,7 +19129,7 @@
         <v>0.214431740824571</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>250</v>
       </c>
@@ -19137,7 +19140,7 @@
         <v>0.21026943516751501</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>251</v>
       </c>
@@ -19148,7 +19151,7 @@
         <v>0.211983108185162</v>
       </c>
     </row>
-    <row r="221" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>252</v>
       </c>
@@ -19159,7 +19162,7 @@
         <v>0.212540414406241</v>
       </c>
     </row>
-    <row r="222" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>253</v>
       </c>
@@ -19170,7 +19173,7 @@
         <v>0.21316933311979799</v>
       </c>
     </row>
-    <row r="223" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>254</v>
       </c>
@@ -19181,7 +19184,7 @@
         <v>0.212515123863107</v>
       </c>
     </row>
-    <row r="224" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>255</v>
       </c>
@@ -19192,7 +19195,7 @@
         <v>0.21030240285409901</v>
       </c>
     </row>
-    <row r="225" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>256</v>
       </c>
@@ -19203,7 +19206,7 @@
         <v>0.213000429148374</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>257</v>
       </c>
@@ -19214,7 +19217,7 @@
         <v>0.21204120218539499</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>258</v>
       </c>
@@ -19225,7 +19228,7 @@
         <v>0.211005527878392</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>259</v>
       </c>
@@ -19236,7 +19239,7 @@
         <v>0.21490935202097999</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>260</v>
       </c>
@@ -19247,7 +19250,7 @@
         <v>0.214705500945685</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>261</v>
       </c>
@@ -19258,7 +19261,7 @@
         <v>0.21046954774395399</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
         <v>262</v>
       </c>
@@ -19269,7 +19272,7 @@
         <v>0.212979730482002</v>
       </c>
     </row>
-    <row r="232" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>263</v>
       </c>
@@ -19280,7 +19283,7 @@
         <v>0.21145441547031901</v>
       </c>
     </row>
-    <row r="233" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
         <v>264</v>
       </c>
@@ -19291,7 +19294,7 @@
         <v>0.21334229216903</v>
       </c>
     </row>
-    <row r="234" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>265</v>
       </c>
@@ -19302,7 +19305,7 @@
         <v>0.21313225436689001</v>
       </c>
     </row>
-    <row r="235" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>266</v>
       </c>
@@ -19313,7 +19316,7 @@
         <v>0.21364986681269199</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
         <v>267</v>
       </c>
@@ -19324,7 +19327,7 @@
         <v>0.21046298569896901</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
         <v>268</v>
       </c>
@@ -19335,7 +19338,7 @@
         <v>0.21370475343700501</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
         <v>269</v>
       </c>
@@ -19346,7 +19349,7 @@
         <v>0.213427613164866</v>
       </c>
     </row>
-    <row r="239" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
         <v>270</v>
       </c>
@@ -19357,7 +19360,7 @@
         <v>0.21285885222227299</v>
       </c>
     </row>
-    <row r="240" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
         <v>271</v>
       </c>
@@ -19368,7 +19371,7 @@
         <v>0.21229610722325801</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
         <v>272</v>
       </c>
@@ -19379,7 +19382,7 @@
         <v>0.213479995323273</v>
       </c>
     </row>
-    <row r="242" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
         <v>244</v>
       </c>
@@ -19390,7 +19393,7 @@
         <v>0.23747635372092801</v>
       </c>
     </row>
-    <row r="243" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
         <v>220</v>
       </c>
@@ -19401,7 +19404,7 @@
         <v>0.24180291421483799</v>
       </c>
     </row>
-    <row r="244" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
         <v>221</v>
       </c>
@@ -19412,7 +19415,7 @@
         <v>0.23775144209915899</v>
       </c>
     </row>
-    <row r="245" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
         <v>222</v>
       </c>
@@ -19423,7 +19426,7 @@
         <v>0.24065215342237201</v>
       </c>
     </row>
-    <row r="246" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
         <v>223</v>
       </c>
@@ -19434,7 +19437,7 @@
         <v>0.238634580986853</v>
       </c>
     </row>
-    <row r="247" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
         <v>224</v>
       </c>
@@ -19445,7 +19448,7 @@
         <v>0.24123516367901099</v>
       </c>
     </row>
-    <row r="248" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
         <v>225</v>
       </c>
@@ -19456,7 +19459,7 @@
         <v>0.23838761262462899</v>
       </c>
     </row>
-    <row r="249" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
         <v>226</v>
       </c>
@@ -19467,7 +19470,7 @@
         <v>0.23787175668006799</v>
       </c>
     </row>
-    <row r="250" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
         <v>227</v>
       </c>
@@ -19478,7 +19481,7 @@
         <v>0.235957408677299</v>
       </c>
     </row>
-    <row r="251" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
         <v>228</v>
       </c>
@@ -19489,7 +19492,7 @@
         <v>0.23761103430247099</v>
       </c>
     </row>
-    <row r="252" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
         <v>229</v>
       </c>
@@ -19500,7 +19503,7 @@
         <v>0.24049928819975</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
         <v>230</v>
       </c>
@@ -19511,7 +19514,7 @@
         <v>0.23875237313230799</v>
       </c>
     </row>
-    <row r="254" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
         <v>231</v>
       </c>
@@ -19522,7 +19525,7 @@
         <v>0.23577509684512599</v>
       </c>
     </row>
-    <row r="255" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
         <v>232</v>
       </c>
@@ -19533,7 +19536,7 @@
         <v>0.23798590162913699</v>
       </c>
     </row>
-    <row r="256" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
         <v>233</v>
       </c>
@@ -19544,7 +19547,7 @@
         <v>0.23776270729380899</v>
       </c>
     </row>
-    <row r="257" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
         <v>234</v>
       </c>
@@ -19555,7 +19558,7 @@
         <v>0.23525871098023601</v>
       </c>
     </row>
-    <row r="258" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
         <v>235</v>
       </c>
@@ -19566,7 +19569,7 @@
         <v>0.23822698567085801</v>
       </c>
     </row>
-    <row r="259" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
         <v>236</v>
       </c>
@@ -19577,7 +19580,7 @@
         <v>0.236137249858582</v>
       </c>
     </row>
-    <row r="260" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
         <v>237</v>
       </c>
@@ -19588,7 +19591,7 @@
         <v>0.236589149526167</v>
       </c>
     </row>
-    <row r="261" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
         <v>238</v>
       </c>
@@ -19599,7 +19602,7 @@
         <v>0.234995035195148</v>
       </c>
     </row>
-    <row r="262" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
         <v>239</v>
       </c>
@@ -19610,7 +19613,7 @@
         <v>0.238435257488993</v>
       </c>
     </row>
-    <row r="263" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
         <v>240</v>
       </c>
@@ -19621,7 +19624,7 @@
         <v>0.23631298859917599</v>
       </c>
     </row>
-    <row r="264" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
         <v>241</v>
       </c>
@@ -19632,7 +19635,7 @@
         <v>0.238968925765909</v>
       </c>
     </row>
-    <row r="265" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
         <v>242</v>
       </c>
@@ -19643,7 +19646,7 @@
         <v>0.237506075673066</v>
       </c>
     </row>
-    <row r="266" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
         <v>243</v>
       </c>
@@ -19654,7 +19657,7 @@
         <v>0.237718713583811</v>
       </c>
     </row>
-    <row r="267" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
         <v>276</v>
       </c>
@@ -19665,7 +19668,7 @@
         <v>0.29193451692567801</v>
       </c>
     </row>
-    <row r="268" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
         <v>277</v>
       </c>
@@ -19676,7 +19679,7 @@
         <v>0.28873287738484599</v>
       </c>
     </row>
-    <row r="269" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
         <v>278</v>
       </c>
@@ -19687,7 +19690,7 @@
         <v>0.28985427653153101</v>
       </c>
     </row>
-    <row r="270" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
         <v>279</v>
       </c>
@@ -19698,7 +19701,7 @@
         <v>0.29473582812057803</v>
       </c>
     </row>
-    <row r="271" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
         <v>280</v>
       </c>
@@ -19709,7 +19712,7 @@
         <v>0.29630016894823502</v>
       </c>
     </row>
-    <row r="272" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
         <v>281</v>
       </c>
@@ -19720,7 +19723,7 @@
         <v>0.290375757335809</v>
       </c>
     </row>
-    <row r="273" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
         <v>282</v>
       </c>
@@ -19731,7 +19734,7 @@
         <v>0.29184259037329402</v>
       </c>
     </row>
-    <row r="274" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
         <v>283</v>
       </c>
@@ -19742,7 +19745,7 @@
         <v>0.29495272762742802</v>
       </c>
     </row>
-    <row r="275" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
         <v>284</v>
       </c>
@@ -19753,7 +19756,7 @@
         <v>0.29546767207366198</v>
       </c>
     </row>
-    <row r="276" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
         <v>285</v>
       </c>
@@ -19764,7 +19767,7 @@
         <v>0.29613521382059799</v>
       </c>
     </row>
-    <row r="277" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
         <v>286</v>
       </c>
@@ -19775,7 +19778,7 @@
         <v>0.29582825670155199</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A278" s="1" t="s">
         <v>287</v>
       </c>
@@ -19786,7 +19789,7 @@
         <v>0.29449530569974303</v>
       </c>
     </row>
-    <row r="279" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
         <v>288</v>
       </c>
@@ -19797,7 +19800,7 @@
         <v>0.29806425275037302</v>
       </c>
     </row>
-    <row r="280" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
         <v>289</v>
       </c>
@@ -19808,7 +19811,7 @@
         <v>0.29361605170472399</v>
       </c>
     </row>
-    <row r="281" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
         <v>290</v>
       </c>
@@ -19819,7 +19822,7 @@
         <v>0.29750345759486801</v>
       </c>
     </row>
-    <row r="282" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
         <v>291</v>
       </c>
@@ -19830,7 +19833,7 @@
         <v>0.29221770492358401</v>
       </c>
     </row>
-    <row r="283" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
         <v>292</v>
       </c>
@@ -19841,7 +19844,7 @@
         <v>0.29462962623990302</v>
       </c>
     </row>
-    <row r="284" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
         <v>293</v>
       </c>
@@ -19852,7 +19855,7 @@
         <v>0.29592312403825599</v>
       </c>
     </row>
-    <row r="285" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A285" s="1" t="s">
         <v>294</v>
       </c>
@@ -19863,7 +19866,7 @@
         <v>0.29448024773360298</v>
       </c>
     </row>
-    <row r="286" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
         <v>295</v>
       </c>
@@ -19874,7 +19877,7 @@
         <v>0.29587930445673999</v>
       </c>
     </row>
-    <row r="287" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
         <v>296</v>
       </c>
@@ -19885,7 +19888,7 @@
         <v>0.28842517989208999</v>
       </c>
     </row>
-    <row r="288" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
         <v>297</v>
       </c>
@@ -19896,7 +19899,7 @@
         <v>0.29360342062414901</v>
       </c>
     </row>
-    <row r="289" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
         <v>298</v>
       </c>
@@ -19907,7 +19910,7 @@
         <v>0.28921987206488498</v>
       </c>
     </row>
-    <row r="290" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
         <v>299</v>
       </c>
@@ -19918,7 +19921,7 @@
         <v>0.29134851176696303</v>
       </c>
     </row>
-    <row r="291" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
         <v>300</v>
       </c>
@@ -19929,7 +19932,7 @@
         <v>0.29264779346075898</v>
       </c>
     </row>
-    <row r="292" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>301</v>
       </c>
@@ -19940,7 +19943,7 @@
         <v>0.28825504808202801</v>
       </c>
     </row>
-    <row r="293" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
         <v>302</v>
       </c>
@@ -19951,7 +19954,7 @@
         <v>0.29422715038680303</v>
       </c>
     </row>
-    <row r="294" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
         <v>303</v>
       </c>
@@ -19962,7 +19965,7 @@
         <v>0.295993095562951</v>
       </c>
     </row>
-    <row r="295" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
         <v>304</v>
       </c>
@@ -19973,7 +19976,7 @@
         <v>0.291643296428021</v>
       </c>
     </row>
-    <row r="296" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
         <v>305</v>
       </c>
@@ -19984,7 +19987,7 @@
         <v>0.29408431924388001</v>
       </c>
     </row>
-    <row r="297" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
         <v>306</v>
       </c>
@@ -20005,13 +20008,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D318508-EB39-4B19-9441-3235666F09D0}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>208</v>
       </c>
@@ -20064,7 +20067,7 @@
         <v>4.8722013994164027E-4</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>209</v>
       </c>
@@ -20117,7 +20120,7 @@
         <v>0.16607519486925235</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>207</v>
       </c>
@@ -20158,7 +20161,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -20199,7 +20202,7 @@
         <v>0.29193451692567801</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -20240,7 +20243,7 @@
         <v>0.28873287738484599</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -20281,7 +20284,7 @@
         <v>0.28985427653153101</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -20322,7 +20325,7 @@
         <v>0.29473582812057803</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -20363,7 +20366,7 @@
         <v>0.29630016894823502</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -20401,7 +20404,7 @@
         <v>0.290375757335809</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -20439,7 +20442,7 @@
         <v>0.29184259037329402</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
@@ -20477,7 +20480,7 @@
         <v>0.29495272762742802</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
@@ -20515,7 +20518,7 @@
         <v>0.29546767207366198</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10</v>
       </c>
@@ -20553,7 +20556,7 @@
         <v>0.29613521382059799</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>11</v>
       </c>
@@ -20591,7 +20594,7 @@
         <v>0.29582825670155199</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>12</v>
       </c>
@@ -20629,7 +20632,7 @@
         <v>0.29449530569974303</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13</v>
       </c>
@@ -20667,7 +20670,7 @@
         <v>0.29806425275037302</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>14</v>
       </c>
@@ -20705,7 +20708,7 @@
         <v>0.29361605170472399</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>15</v>
       </c>
@@ -20743,7 +20746,7 @@
         <v>0.29750345759486801</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>16</v>
       </c>
@@ -20778,7 +20781,7 @@
         <v>0.29221770492358401</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>17</v>
       </c>
@@ -20810,7 +20813,7 @@
         <v>0.29462962623990302</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>18</v>
       </c>
@@ -20842,7 +20845,7 @@
         <v>0.29592312403825599</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>19</v>
       </c>
@@ -20874,7 +20877,7 @@
         <v>0.29448024773360298</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>20</v>
       </c>
@@ -20903,7 +20906,7 @@
         <v>0.29587930445673999</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>21</v>
       </c>
@@ -20929,7 +20932,7 @@
         <v>0.28842517989208999</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>22</v>
       </c>
@@ -20955,7 +20958,7 @@
         <v>0.29360342062414901</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
@@ -20981,7 +20984,7 @@
         <v>0.28921987206488498</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
@@ -21004,7 +21007,7 @@
         <v>0.29134851176696303</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
@@ -21027,7 +21030,7 @@
         <v>0.29264779346075898</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>26</v>
       </c>
@@ -21050,7 +21053,7 @@
         <v>0.28825504808202801</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>27</v>
       </c>
@@ -21073,7 +21076,7 @@
         <v>0.29422715038680303</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>28</v>
       </c>
@@ -21096,7 +21099,7 @@
         <v>0.295993095562951</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>29</v>
       </c>
@@ -21116,7 +21119,7 @@
         <v>0.291643296428021</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30</v>
       </c>
@@ -21136,7 +21139,7 @@
         <v>0.29408431924388001</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>31</v>
       </c>
@@ -21156,7 +21159,7 @@
         <v>0.29215304331091801</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>32</v>
       </c>
@@ -21167,7 +21170,7 @@
         <v>0.22249606599096799</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>33</v>
       </c>
@@ -21175,7 +21178,7 @@
         <v>0.22770140189949001</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>34</v>
       </c>
@@ -21183,7 +21186,7 @@
         <v>0.22467693879523801</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>35</v>
       </c>
@@ -21191,7 +21194,7 @@
         <v>0.22590951148508701</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>36</v>
       </c>
@@ -21209,12 +21212,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A5AE877-64C3-4028-8147-765389663D58}">
   <dimension ref="A1:M39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>208</v>
       </c>
@@ -21267,7 +21270,7 @@
         <v>1.5436675245504185E-2</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>209</v>
       </c>
@@ -21320,7 +21323,7 @@
         <v>8.55645429483185E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>207</v>
       </c>
@@ -21361,7 +21364,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -21402,7 +21405,7 @@
         <v>17.825013007136501</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -21443,7 +21446,7 @@
         <v>17.9319730766783</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -21484,7 +21487,7 @@
         <v>18.039044650769</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -21525,7 +21528,7 @@
         <v>18.0604756933053</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -21566,7 +21569,7 @@
         <v>17.9979172106978</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -21604,7 +21607,7 @@
         <v>17.998827423434999</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -21642,7 +21645,7 @@
         <v>18.041509768701101</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
@@ -21680,7 +21683,7 @@
         <v>18.113057907959</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
@@ -21718,7 +21721,7 @@
         <v>18.000340035364701</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10</v>
       </c>
@@ -21756,7 +21759,7 @@
         <v>18.056008326627001</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>11</v>
       </c>
@@ -21794,7 +21797,7 @@
         <v>18.143480906181601</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>12</v>
       </c>
@@ -21832,7 +21835,7 @@
         <v>18.0505063076521</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13</v>
       </c>
@@ -21870,7 +21873,7 @@
         <v>17.975837914720699</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>14</v>
       </c>
@@ -21908,7 +21911,7 @@
         <v>17.958408612980101</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>15</v>
       </c>
@@ -21946,7 +21949,7 @@
         <v>18.089794941394199</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>16</v>
       </c>
@@ -21981,7 +21984,7 @@
         <v>18.011107051113001</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>17</v>
       </c>
@@ -22013,7 +22016,7 @@
         <v>18.059805482066999</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>18</v>
       </c>
@@ -22045,7 +22048,7 @@
         <v>17.9483749982906</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>19</v>
       </c>
@@ -22077,7 +22080,7 @@
         <v>17.986594818813899</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>20</v>
       </c>
@@ -22106,7 +22109,7 @@
         <v>18.0136321630971</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>21</v>
       </c>
@@ -22132,7 +22135,7 @@
         <v>18.175378572568899</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>22</v>
       </c>
@@ -22158,7 +22161,7 @@
         <v>18.118575471661899</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
@@ -22184,7 +22187,7 @@
         <v>17.929983986435602</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
@@ -22207,7 +22210,7 @@
         <v>18.106604307150199</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
@@ -22230,7 +22233,7 @@
         <v>17.996855885347902</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>26</v>
       </c>
@@ -22253,7 +22256,7 @@
         <v>18.121396667491499</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>27</v>
       </c>
@@ -22276,7 +22279,7 @@
         <v>18.094216738234799</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>28</v>
       </c>
@@ -22299,7 +22302,7 @@
         <v>18.1174045096291</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>29</v>
       </c>
@@ -22319,7 +22322,7 @@
         <v>17.975345051957699</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>30</v>
       </c>
@@ -22339,7 +22342,7 @@
         <v>18.0641154539816</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>31</v>
       </c>
@@ -22359,7 +22362,7 @@
         <v>18.268545430641002</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>32</v>
       </c>
@@ -22370,7 +22373,7 @@
         <v>13.9597270287277</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>33</v>
       </c>
@@ -22378,7 +22381,7 @@
         <v>13.946102058433601</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>34</v>
       </c>
@@ -22386,7 +22389,7 @@
         <v>13.9823014618208</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>35</v>
       </c>
@@ -22394,7 +22397,7 @@
         <v>13.749906400784599</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
Need to rerun for F1=4
</commit_message>
<xml_diff>
--- a/Fit Results/AllFitsF1=3.xlsx
+++ b/Fit Results/AllFitsF1=3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\Fit Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C37905-4062-4D15-ABB2-40EBDEB099B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A179A515-3971-45BB-BD0D-85A5D926BCCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Together" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="375">
   <si>
     <t>Date</t>
   </si>
@@ -987,6 +987,183 @@
   </si>
   <si>
     <t>Jun09,2026+4-42-24PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-04-00PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-13-10PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-22-33PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-30-33PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-38-38PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-46-37PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+3-54-53PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+4-02-52PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+4-11-03PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+4-19-02PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+4-29-19PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+4-38-38PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+4-50-06PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+5-14-19PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+5-22-17PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+5-34-47PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+5-42-51PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+6-20-54PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+6-35-34PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+6-43-28PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+6-52-08PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+7-09-53PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+7-17-49PM</t>
+  </si>
+  <si>
+    <t>Jul15,2026+7-27-51PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+8-55-13AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-04-11AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-15-02AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-23-01AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-33-02AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-41-08AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-49-15AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+9-57-53AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+10-05-58AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+10-14-09AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+10-22-13AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+10-30-40AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+10-39-15AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+10-47-37AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+11-01-11AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+11-09-27AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+11-17-25AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+11-25-19AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+11-36-19AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+11-44-18AM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+12-12-00PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+12-19-52PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+12-38-41PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+12-47-04PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+12-55-34PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-03-40PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-12-17PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-21-11PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-29-15PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-38-48PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-49-33PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+1-57-55PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+2-05-51PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+2-33-57PM</t>
+  </si>
+  <si>
+    <t>Jul16,2026+3-07-41PM</t>
   </si>
 </sst>
 </file>
@@ -5809,6 +5986,478 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-E80C-4167-B4B8-8BD422FACC58}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="13"/>
+          <c:order val="13"/>
+          <c:tx>
+            <c:v>15-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'All Together'!$B$298:$B$321</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>5.2401573655099698</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.2402095305102501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.2325481598897898</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.2632048700287699</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.2341542225512701</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.2499074678307798</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.2609478156281302</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.2522638411999596</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.2381148673874796</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.2236574261532196</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.2262449444555799</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.2457271314303799</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.2597760818477397</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.2273625593786797</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>5.2281725990355099</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.2464873820867899</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.2357499987829099</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.2426137496126399</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.25389374708476</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.2452132048918996</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>5.2477036957110901</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>5.1912280334424699</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>5.2649162726060403</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>5.2682959002266401</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'All Together'!$C$298:$C$321</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="24"/>
+                <c:pt idx="0">
+                  <c:v>0.10788210556906901</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.107767689685955</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.1085661885666</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.107813849166461</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.10768118552928301</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.10798815957236201</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.10796561723725399</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.107310696139959</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.107235378128852</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.107380313151722</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.107499657333732</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.107395325995434</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.107617315330632</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.107631821742582</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.107773221003444</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.108054680115061</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.108470442647848</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.108306765636387</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.10817681982411</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.107850584510117</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.108220094487482</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.107772509976481</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.108972267405539</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.107940873985824</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3942-410D-8CB2-0AE8962B2BB7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="14"/>
+          <c:order val="14"/>
+          <c:tx>
+            <c:v>16-Jul</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="80000"/>
+                  <a:lumOff val="20000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="80000"/>
+                    <a:lumOff val="20000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'All Together'!$B$322:$B$356</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="35"/>
+                <c:pt idx="0">
+                  <c:v>4.0504847360743401</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0496768121653703</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.0401570007949097</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.0452933053436704</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.0393053513377497</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.0427869051265404</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.0371132630075302</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.0301105995964903</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.0520999190004696</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.0532303423785203</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.0597656945719098</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.0397313521665303</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.0389446603470498</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.0491521884945199</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.0282207799584802</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4.0373666399902799</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4.0254616281370303</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4.0346044905874798</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4.0220126763814203</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.0377589881580498</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>4.0016969711271004</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.9850777599500198</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>4.0132441168710704</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>4.0107044449171996</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4.0042080560711302</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>4.0137738076926297</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>4.0189067438591497</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4.0019418304313801</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>4.0058057955871602</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>4.0060301681826802</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3.99829105994908</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3.9906830558389799</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3.99736506566357</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>3.98390122498571</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>3.9792620371784699</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'All Together'!$C$322:$C$356</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="35"/>
+                <c:pt idx="0">
+                  <c:v>8.3156282475135901E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.3308052923752804E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.3192433829034101E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.3623706474663606E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.3216917778572402E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.3221177215463099E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.33781973276186E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.33668584997104E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.2653296245640703E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8.3314551683197596E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8.3433338441133195E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8.3208643584929701E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.3420473796778499E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8.3107161558914899E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8.3039185267029303E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8.3538722608662797E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8.3535910062118204E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8.3082835466929905E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8.3201985411368501E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8.3110318912883605E-2</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>8.2031859042136696E-2</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>8.2441921487811098E-2</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>8.2431599113651E-2</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>8.3008569433927301E-2</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>8.2766374795728306E-2</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>8.2788867848109599E-2</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>8.3275717539275304E-2</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>8.2647130527365498E-2</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>8.2574146110371893E-2</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>8.23716711721698E-2</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>8.2532915515358393E-2</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>8.2694298166149094E-2</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>8.2670956206444698E-2</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>8.1803833529134007E-2</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>8.1619568336985804E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-3942-410D-8CB2-0AE8962B2BB7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -16613,7 +17262,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R297"/>
+  <dimension ref="A1:R356"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="16.140625" customWidth="1"/>
@@ -16649,7 +17298,7 @@
       </c>
       <c r="E2">
         <f>COUNT(B:B)</f>
-        <v>293</v>
+        <v>352</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>206</v>
@@ -19996,6 +20645,655 @@
       </c>
       <c r="C297" s="1">
         <v>0.29215304331091801</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A298" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B298" s="1">
+        <v>5.2401573655099698</v>
+      </c>
+      <c r="C298" s="1">
+        <v>0.10788210556906901</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A299" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B299" s="1">
+        <v>5.2402095305102501</v>
+      </c>
+      <c r="C299" s="1">
+        <v>0.107767689685955</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A300" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B300" s="1">
+        <v>5.2325481598897898</v>
+      </c>
+      <c r="C300" s="1">
+        <v>0.1085661885666</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A301" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B301" s="1">
+        <v>5.2632048700287699</v>
+      </c>
+      <c r="C301" s="1">
+        <v>0.107813849166461</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A302" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="B302" s="1">
+        <v>5.2341542225512701</v>
+      </c>
+      <c r="C302" s="1">
+        <v>0.10768118552928301</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A303" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B303" s="1">
+        <v>5.2499074678307798</v>
+      </c>
+      <c r="C303" s="1">
+        <v>0.10798815957236201</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A304" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="B304" s="1">
+        <v>5.2609478156281302</v>
+      </c>
+      <c r="C304" s="1">
+        <v>0.10796561723725399</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A305" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B305" s="1">
+        <v>5.2522638411999596</v>
+      </c>
+      <c r="C305" s="1">
+        <v>0.107310696139959</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A306" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B306" s="1">
+        <v>5.2381148673874796</v>
+      </c>
+      <c r="C306" s="1">
+        <v>0.107235378128852</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A307" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B307" s="1">
+        <v>5.2236574261532196</v>
+      </c>
+      <c r="C307" s="1">
+        <v>0.107380313151722</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A308" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B308" s="1">
+        <v>5.2262449444555799</v>
+      </c>
+      <c r="C308" s="1">
+        <v>0.107499657333732</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A309" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B309" s="1">
+        <v>5.2457271314303799</v>
+      </c>
+      <c r="C309" s="1">
+        <v>0.107395325995434</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A310" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B310" s="1">
+        <v>5.2597760818477397</v>
+      </c>
+      <c r="C310" s="1">
+        <v>0.107617315330632</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A311" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B311" s="1">
+        <v>5.2273625593786797</v>
+      </c>
+      <c r="C311" s="1">
+        <v>0.107631821742582</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A312" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B312" s="1">
+        <v>5.2281725990355099</v>
+      </c>
+      <c r="C312" s="1">
+        <v>0.107773221003444</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A313" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B313" s="1">
+        <v>5.2464873820867899</v>
+      </c>
+      <c r="C313" s="1">
+        <v>0.108054680115061</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A314" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B314" s="1">
+        <v>5.2357499987829099</v>
+      </c>
+      <c r="C314" s="1">
+        <v>0.108470442647848</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A315" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="B315" s="1">
+        <v>5.2426137496126399</v>
+      </c>
+      <c r="C315" s="1">
+        <v>0.108306765636387</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A316" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B316" s="1">
+        <v>5.25389374708476</v>
+      </c>
+      <c r="C316" s="1">
+        <v>0.10817681982411</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A317" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B317" s="1">
+        <v>5.2452132048918996</v>
+      </c>
+      <c r="C317" s="1">
+        <v>0.107850584510117</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A318" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B318" s="1">
+        <v>5.2477036957110901</v>
+      </c>
+      <c r="C318" s="1">
+        <v>0.108220094487482</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A319" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B319" s="1">
+        <v>5.1912280334424699</v>
+      </c>
+      <c r="C319" s="1">
+        <v>0.107772509976481</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A320" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="B320" s="1">
+        <v>5.2649162726060403</v>
+      </c>
+      <c r="C320" s="1">
+        <v>0.108972267405539</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A321" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B321" s="1">
+        <v>5.2682959002266401</v>
+      </c>
+      <c r="C321" s="1">
+        <v>0.107940873985824</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A322" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B322" s="1">
+        <v>4.0504847360743401</v>
+      </c>
+      <c r="C322" s="1">
+        <v>8.3156282475135901E-2</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A323" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B323" s="1">
+        <v>4.0496768121653703</v>
+      </c>
+      <c r="C323" s="1">
+        <v>8.3308052923752804E-2</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A324" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B324" s="1">
+        <v>4.0401570007949097</v>
+      </c>
+      <c r="C324" s="1">
+        <v>8.3192433829034101E-2</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A325" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B325" s="1">
+        <v>4.0452933053436704</v>
+      </c>
+      <c r="C325" s="1">
+        <v>8.3623706474663606E-2</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A326" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B326" s="1">
+        <v>4.0393053513377497</v>
+      </c>
+      <c r="C326" s="1">
+        <v>8.3216917778572402E-2</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A327" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B327" s="1">
+        <v>4.0427869051265404</v>
+      </c>
+      <c r="C327" s="1">
+        <v>8.3221177215463099E-2</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A328" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B328" s="1">
+        <v>4.0371132630075302</v>
+      </c>
+      <c r="C328" s="1">
+        <v>8.33781973276186E-2</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A329" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B329" s="1">
+        <v>4.0301105995964903</v>
+      </c>
+      <c r="C329" s="1">
+        <v>8.33668584997104E-2</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A330" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B330" s="1">
+        <v>4.0520999190004696</v>
+      </c>
+      <c r="C330" s="1">
+        <v>8.2653296245640703E-2</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A331" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B331" s="1">
+        <v>4.0532303423785203</v>
+      </c>
+      <c r="C331" s="1">
+        <v>8.3314551683197596E-2</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A332" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B332" s="1">
+        <v>4.0597656945719098</v>
+      </c>
+      <c r="C332" s="1">
+        <v>8.3433338441133195E-2</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A333" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B333" s="1">
+        <v>4.0397313521665303</v>
+      </c>
+      <c r="C333" s="1">
+        <v>8.3208643584929701E-2</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A334" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B334" s="1">
+        <v>4.0389446603470498</v>
+      </c>
+      <c r="C334" s="1">
+        <v>8.3420473796778499E-2</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A335" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B335" s="1">
+        <v>4.0491521884945199</v>
+      </c>
+      <c r="C335" s="1">
+        <v>8.3107161558914899E-2</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A336" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B336" s="1">
+        <v>4.0282207799584802</v>
+      </c>
+      <c r="C336" s="1">
+        <v>8.3039185267029303E-2</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A337" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B337" s="1">
+        <v>4.0373666399902799</v>
+      </c>
+      <c r="C337" s="1">
+        <v>8.3538722608662797E-2</v>
+      </c>
+    </row>
+    <row r="338" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A338" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B338" s="1">
+        <v>4.0254616281370303</v>
+      </c>
+      <c r="C338" s="1">
+        <v>8.3535910062118204E-2</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A339" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B339" s="1">
+        <v>4.0346044905874798</v>
+      </c>
+      <c r="C339" s="1">
+        <v>8.3082835466929905E-2</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A340" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B340" s="1">
+        <v>4.0220126763814203</v>
+      </c>
+      <c r="C340" s="1">
+        <v>8.3201985411368501E-2</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A341" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B341" s="1">
+        <v>4.0377589881580498</v>
+      </c>
+      <c r="C341" s="1">
+        <v>8.3110318912883605E-2</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A342" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B342" s="1">
+        <v>4.0016969711271004</v>
+      </c>
+      <c r="C342" s="1">
+        <v>8.2031859042136696E-2</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A343" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B343" s="1">
+        <v>3.9850777599500198</v>
+      </c>
+      <c r="C343" s="1">
+        <v>8.2441921487811098E-2</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A344" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B344" s="1">
+        <v>4.0132441168710704</v>
+      </c>
+      <c r="C344" s="1">
+        <v>8.2431599113651E-2</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A345" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B345" s="1">
+        <v>4.0107044449171996</v>
+      </c>
+      <c r="C345" s="1">
+        <v>8.3008569433927301E-2</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A346" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B346" s="1">
+        <v>4.0042080560711302</v>
+      </c>
+      <c r="C346" s="1">
+        <v>8.2766374795728306E-2</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A347" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B347" s="1">
+        <v>4.0137738076926297</v>
+      </c>
+      <c r="C347" s="1">
+        <v>8.2788867848109599E-2</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A348" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B348" s="1">
+        <v>4.0189067438591497</v>
+      </c>
+      <c r="C348" s="1">
+        <v>8.3275717539275304E-2</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A349" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B349" s="1">
+        <v>4.0019418304313801</v>
+      </c>
+      <c r="C349" s="1">
+        <v>8.2647130527365498E-2</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A350" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B350" s="1">
+        <v>4.0058057955871602</v>
+      </c>
+      <c r="C350" s="1">
+        <v>8.2574146110371893E-2</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A351" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B351" s="1">
+        <v>4.0060301681826802</v>
+      </c>
+      <c r="C351" s="1">
+        <v>8.23716711721698E-2</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A352" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B352" s="1">
+        <v>3.99829105994908</v>
+      </c>
+      <c r="C352" s="1">
+        <v>8.2532915515358393E-2</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A353" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B353" s="1">
+        <v>3.9906830558389799</v>
+      </c>
+      <c r="C353" s="1">
+        <v>8.2694298166149094E-2</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A354" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B354" s="1">
+        <v>3.99736506566357</v>
+      </c>
+      <c r="C354" s="1">
+        <v>8.2670956206444698E-2</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A355" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="B355" s="1">
+        <v>3.98390122498571</v>
+      </c>
+      <c r="C355" s="1">
+        <v>8.1803833529134007E-2</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A356" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B356" s="1">
+        <v>3.9792620371784699</v>
+      </c>
+      <c r="C356" s="1">
+        <v>8.1619568336985804E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>